<commit_message>
updated reg_estimates remaining estimates to be updated are: -reg_education.xlsx -reg_labourSupplyUtility.xlsx
</commit_message>
<xml_diff>
--- a/input/ES/reg_home_ownership.xlsx
+++ b/input/ES/reg_home_ownership.xlsx
@@ -508,100 +508,100 @@
         <v>0.00044992553030662381</v>
       </c>
       <c r="D2">
-        <v>8.5196106026390415e-05</v>
+        <v>8.5196106026389927e-05</v>
       </c>
       <c r="E2">
-        <v>-6.2828630875756437e-05</v>
+        <v>-6.2828630875756355e-05</v>
       </c>
       <c r="F2">
-        <v>-8.4565668852782602e-06</v>
+        <v>-8.4565668852783889e-06</v>
       </c>
       <c r="G2">
-        <v>-0.00010843423021864615</v>
+        <v>-0.00010843423021864604</v>
       </c>
       <c r="H2">
-        <v>-0.00010596516053969346</v>
+        <v>-0.00010596516053969373</v>
       </c>
       <c r="I2">
-        <v>0.00011732840928461018</v>
+        <v>0.00011732840928460902</v>
       </c>
       <c r="J2">
-        <v>0.00018803916794095022</v>
+        <v>0.00018803916794095035</v>
       </c>
       <c r="K2">
-        <v>5.1197771764598007e-06</v>
+        <v>5.1197771764612237e-06</v>
       </c>
       <c r="L2">
-        <v>-4.2400694082288633e-05</v>
+        <v>-4.2400694082287739e-05</v>
       </c>
       <c r="M2">
-        <v>-6.0906119824910346e-05</v>
+        <v>-6.0906119824910264e-05</v>
       </c>
       <c r="N2">
-        <v>-3.361322185230121e-05</v>
+        <v>-3.3613221852301075e-05</v>
       </c>
       <c r="O2">
-        <v>-4.8211227158035332e-05</v>
+        <v>-4.8211227158035095e-05</v>
       </c>
       <c r="P2">
-        <v>0.00015964187899656531</v>
+        <v>0.00015964187899656515</v>
       </c>
       <c r="Q2">
-        <v>-2.9367506558327801e-05</v>
+        <v>-2.9367506558323816e-05</v>
       </c>
       <c r="R2">
-        <v>-5.3783345333062307e-05</v>
+        <v>-5.3783345333062239e-05</v>
       </c>
       <c r="S2">
-        <v>-0.00011313088460214999</v>
+        <v>-0.00011313088460214739</v>
       </c>
       <c r="T2">
-        <v>3.3585706080962048e-07</v>
+        <v>3.3585706081016427e-07</v>
       </c>
       <c r="U2">
-        <v>3.897800193710734e-05</v>
+        <v>3.8978001937107882e-05</v>
       </c>
       <c r="V2">
-        <v>-1.429762836629479e-06</v>
+        <v>-1.4297628366294248e-06</v>
       </c>
       <c r="W2">
-        <v>-5.9422502834602001e-05</v>
+        <v>-5.9422502834600118e-05</v>
       </c>
       <c r="X2">
-        <v>-4.802813257907438e-07</v>
+        <v>-4.8028132579072198e-07</v>
       </c>
       <c r="Y2">
-        <v>-3.1834493471115892e-05</v>
+        <v>-3.1834493471115865e-05</v>
       </c>
       <c r="Z2">
-        <v>-8.1085924364915341e-05</v>
+        <v>-8.1085924364914826e-05</v>
       </c>
       <c r="AA2">
-        <v>-8.7021960423897996e-05</v>
+        <v>-8.7021960423897508e-05</v>
       </c>
       <c r="AB2">
-        <v>-9.2596972208624484e-05</v>
+        <v>-9.2596972208624809e-05</v>
       </c>
       <c r="AC2">
-        <v>-0.00010856841590938738</v>
+        <v>-0.00010856841590938695</v>
       </c>
       <c r="AD2">
-        <v>-6.3819334106375331e-05</v>
+        <v>-6.3819334106375602e-05</v>
       </c>
       <c r="AE2">
-        <v>-4.7641209485684455e-06</v>
+        <v>-4.7641209485679661e-06</v>
       </c>
       <c r="AF2">
-        <v>-1.9497710287320405e-06</v>
+        <v>-1.9497710287320125e-06</v>
       </c>
       <c r="AG2">
-        <v>8.2682461790918376e-05</v>
+        <v>8.2682461790918268e-05</v>
       </c>
       <c r="AH2">
-        <v>1.3097791130418853e-05</v>
+        <v>1.3097791130418568e-05</v>
       </c>
       <c r="AI2">
-        <v>-7.2034827626274e-05</v>
+        <v>-7.2034827626278066e-05</v>
       </c>
     </row>
     <row r="3">
@@ -612,103 +612,103 @@
         <v>0.12681895963208956</v>
       </c>
       <c r="C3">
-        <v>8.5196106026390415e-05</v>
+        <v>8.5196106026389927e-05</v>
       </c>
       <c r="D3">
         <v>0.15220756463936075</v>
       </c>
       <c r="E3">
-        <v>0.002084396923760304</v>
+        <v>0.0020843969237603283</v>
       </c>
       <c r="F3">
-        <v>0.0016882452590596976</v>
+        <v>0.0016882452590597011</v>
       </c>
       <c r="G3">
-        <v>0.0024417879512849943</v>
+        <v>0.0024417879512850195</v>
       </c>
       <c r="H3">
-        <v>0.0021134510801234059</v>
+        <v>0.0021134510801234241</v>
       </c>
       <c r="I3">
-        <v>0.0019828406336588871</v>
+        <v>0.0019828406336589123</v>
       </c>
       <c r="J3">
-        <v>0.0020871683533679178</v>
+        <v>0.0020871683533679438</v>
       </c>
       <c r="K3">
-        <v>-2.0115308488022473e-05</v>
+        <v>-2.0115308488016619e-05</v>
       </c>
       <c r="L3">
-        <v>0.0001862923207223158</v>
+        <v>0.0001862923207223358</v>
       </c>
       <c r="M3">
-        <v>0.00027309987750996157</v>
+        <v>0.00027309987750996309</v>
       </c>
       <c r="N3">
-        <v>3.415495757352156e-05</v>
+        <v>3.4154957573525626e-05</v>
       </c>
       <c r="O3">
-        <v>0.00017304750110305124</v>
+        <v>0.00017304750110305598</v>
       </c>
       <c r="P3">
-        <v>0.00024098226622748672</v>
+        <v>0.00024098226622749843</v>
       </c>
       <c r="Q3">
-        <v>0.0002049088881617481</v>
+        <v>0.00020490888816182367</v>
       </c>
       <c r="R3">
-        <v>0.00013961429365073885</v>
+        <v>0.00013961429365074959</v>
       </c>
       <c r="S3">
-        <v>0.00035347518107974138</v>
+        <v>0.00035347518107978909</v>
       </c>
       <c r="T3">
-        <v>-1.9174180004394734e-05</v>
+        <v>-1.9174180004385085e-05</v>
       </c>
       <c r="U3">
-        <v>-3.2793598063826689e-05</v>
+        <v>-3.2793598063814329e-05</v>
       </c>
       <c r="V3">
-        <v>0.00034904637853419248</v>
+        <v>0.00034904637853420397</v>
       </c>
       <c r="W3">
-        <v>0.00080519745304555952</v>
+        <v>0.000805197453045594</v>
       </c>
       <c r="X3">
-        <v>-7.8230614138234162e-06</v>
+        <v>-7.8230614138232163e-06</v>
       </c>
       <c r="Y3">
-        <v>0.00033228372241895826</v>
+        <v>0.00033228372241895908</v>
       </c>
       <c r="Z3">
-        <v>0.00014280146279554637</v>
+        <v>0.00014280146279555895</v>
       </c>
       <c r="AA3">
-        <v>0.0010716454027064866</v>
+        <v>0.0010716454027064983</v>
       </c>
       <c r="AB3">
-        <v>0.0007563371623317567</v>
+        <v>0.0007563371623317696</v>
       </c>
       <c r="AC3">
-        <v>0.00013931877986970488</v>
+        <v>0.00013931877986971463</v>
       </c>
       <c r="AD3">
-        <v>0.00013819997115470237</v>
+        <v>0.0001381999711547124</v>
       </c>
       <c r="AE3">
-        <v>2.6842920995643992e-05</v>
+        <v>2.6842920995656433e-05</v>
       </c>
       <c r="AF3">
-        <v>-8.510155342639439e-06</v>
+        <v>-8.510155342638653e-06</v>
       </c>
       <c r="AG3">
-        <v>5.4247913094004809e-05</v>
+        <v>5.4247913094002641e-05</v>
       </c>
       <c r="AH3">
-        <v>0.0013306349657106415</v>
+        <v>0.0013306349657106369</v>
       </c>
       <c r="AI3">
-        <v>-0.0029610538351407139</v>
+        <v>-0.0029610538351408063</v>
       </c>
     </row>
     <row r="4">
@@ -719,103 +719,103 @@
         <v>0.03595234274131201</v>
       </c>
       <c r="C4">
-        <v>-6.2828630875756437e-05</v>
+        <v>-6.2828630875756355e-05</v>
       </c>
       <c r="D4">
-        <v>0.002084396923760304</v>
+        <v>0.0020843969237603283</v>
       </c>
       <c r="E4">
-        <v>0.0026441163376976526</v>
+        <v>0.0026441163376976738</v>
       </c>
       <c r="F4">
-        <v>0.0018128197573376338</v>
+        <v>0.0018128197573376375</v>
       </c>
       <c r="G4">
-        <v>0.0020642741812237952</v>
+        <v>0.0020642741812238186</v>
       </c>
       <c r="H4">
-        <v>0.0020977832497201653</v>
+        <v>0.0020977832497201827</v>
       </c>
       <c r="I4">
-        <v>0.0021085718188296109</v>
+        <v>0.0021085718188296331</v>
       </c>
       <c r="J4">
-        <v>0.0021090443932507389</v>
+        <v>0.0021090443932507631</v>
       </c>
       <c r="K4">
-        <v>1.4118593225045939e-05</v>
+        <v>1.4118593225052661e-05</v>
       </c>
       <c r="L4">
-        <v>-9.3260023870279937e-05</v>
+        <v>-9.3260023870260489e-05</v>
       </c>
       <c r="M4">
-        <v>0.00011537275032906199</v>
+        <v>0.00011537275032906373</v>
       </c>
       <c r="N4">
-        <v>0.00013157663846053444</v>
+        <v>0.00013157663846053829</v>
       </c>
       <c r="O4">
-        <v>9.2101658019669966e-05</v>
+        <v>9.2101658019674547e-05</v>
       </c>
       <c r="P4">
-        <v>0.00025685583857601392</v>
+        <v>0.00025685583857602715</v>
       </c>
       <c r="Q4">
-        <v>7.6911989027215739e-05</v>
+        <v>7.6911989027287839e-05</v>
       </c>
       <c r="R4">
-        <v>5.8410909162380639e-05</v>
+        <v>5.8410909162392619e-05</v>
       </c>
       <c r="S4">
-        <v>0.00011723908016807649</v>
+        <v>0.00011723908016812289</v>
       </c>
       <c r="T4">
-        <v>7.8675240484065185e-05</v>
+        <v>7.8675240484074415e-05</v>
       </c>
       <c r="U4">
-        <v>9.0123156531705896e-05</v>
+        <v>9.0123156531717605e-05</v>
       </c>
       <c r="V4">
-        <v>0.00023564401616686876</v>
+        <v>0.00023564401616688263</v>
       </c>
       <c r="W4">
-        <v>0.00072939579332476838</v>
+        <v>0.0007293957933247996</v>
       </c>
       <c r="X4">
-        <v>-3.1864712784610305e-05</v>
+        <v>-3.1864712784610176e-05</v>
       </c>
       <c r="Y4">
-        <v>-6.7136134926304263e-05</v>
+        <v>-6.7136134926303558e-05</v>
       </c>
       <c r="Z4">
-        <v>0.00010394145986337652</v>
+        <v>0.00010394145986338931</v>
       </c>
       <c r="AA4">
-        <v>8.770373819365785e-05</v>
+        <v>8.7703738193669126e-05</v>
       </c>
       <c r="AB4">
-        <v>0.00010743254938749445</v>
+        <v>0.00010743254938750703</v>
       </c>
       <c r="AC4">
-        <v>4.3360577271745913e-05</v>
+        <v>4.3360577271755454e-05</v>
       </c>
       <c r="AD4">
-        <v>6.5902518832273212e-05</v>
+        <v>6.5902518832282645e-05</v>
       </c>
       <c r="AE4">
-        <v>-1.1316323787113696e-05</v>
+        <v>-1.1316323787101472e-05</v>
       </c>
       <c r="AF4">
-        <v>5.5397297790903439e-06</v>
+        <v>5.5397297790910622e-06</v>
       </c>
       <c r="AG4">
-        <v>-3.4781742681625188e-05</v>
+        <v>-3.478174268162779e-05</v>
       </c>
       <c r="AH4">
-        <v>2.948272168971347e-05</v>
+        <v>2.9482721689708916e-05</v>
       </c>
       <c r="AI4">
-        <v>-0.0024047977311919084</v>
+        <v>-0.0024047977311919999</v>
       </c>
     </row>
     <row r="5">
@@ -826,103 +826,103 @@
         <v>-0.076810395035844345</v>
       </c>
       <c r="C5">
-        <v>-8.4565668852782602e-06</v>
+        <v>-8.4565668852783889e-06</v>
       </c>
       <c r="D5">
-        <v>0.0016882452590596976</v>
+        <v>0.0016882452590597011</v>
       </c>
       <c r="E5">
-        <v>0.0018128197573376338</v>
+        <v>0.0018128197573376375</v>
       </c>
       <c r="F5">
-        <v>0.0028941737281210798</v>
+        <v>0.0028941737281210829</v>
       </c>
       <c r="G5">
-        <v>0.0018612724534218567</v>
+        <v>0.0018612724534218779</v>
       </c>
       <c r="H5">
-        <v>0.0018492289694546063</v>
+        <v>0.0018492289694546213</v>
       </c>
       <c r="I5">
-        <v>0.001802882282930145</v>
+        <v>0.001802882282930165</v>
       </c>
       <c r="J5">
-        <v>0.0017667256002488313</v>
+        <v>0.0017667256002488528</v>
       </c>
       <c r="K5">
-        <v>0.0001037959055400241</v>
+        <v>0.00010379590554003039</v>
       </c>
       <c r="L5">
-        <v>9.6185840505532403e-05</v>
+        <v>9.6185840505550211e-05</v>
       </c>
       <c r="M5">
-        <v>8.1680466308312917e-05</v>
+        <v>8.1680466308314218e-05</v>
       </c>
       <c r="N5">
-        <v>0.00012419560983464682</v>
+        <v>0.00012419560983465032</v>
       </c>
       <c r="O5">
-        <v>0.00011222399271491033</v>
+        <v>0.00011222399271491425</v>
       </c>
       <c r="P5">
-        <v>2.6036874602798177e-05</v>
+        <v>2.6036874602808802e-05</v>
       </c>
       <c r="Q5">
-        <v>3.0606587825475549e-05</v>
+        <v>3.0606587825537783e-05</v>
       </c>
       <c r="R5">
-        <v>-5.2813169843047366e-06</v>
+        <v>-5.2813169842945993e-06</v>
       </c>
       <c r="S5">
-        <v>2.2049062175248733e-05</v>
+        <v>2.2049062175289933e-05</v>
       </c>
       <c r="T5">
-        <v>3.3185996693455404e-05</v>
+        <v>3.3185996693463644e-05</v>
       </c>
       <c r="U5">
-        <v>4.759201680919038e-05</v>
+        <v>4.7592016809201655e-05</v>
       </c>
       <c r="V5">
-        <v>6.0529809378991268e-05</v>
+        <v>6.0529809379003194e-05</v>
       </c>
       <c r="W5">
-        <v>0.00035402050081689601</v>
+        <v>0.00035402050081692485</v>
       </c>
       <c r="X5">
-        <v>-1.1239453734116289e-05</v>
+        <v>-1.1239453734116243e-05</v>
       </c>
       <c r="Y5">
-        <v>-4.883454486433441e-05</v>
+        <v>-4.883454486433376e-05</v>
       </c>
       <c r="Z5">
-        <v>0.00011191749201079561</v>
+        <v>0.00011191749201080623</v>
       </c>
       <c r="AA5">
-        <v>7.3842847933200395e-06</v>
+        <v>7.3842847933297973e-06</v>
       </c>
       <c r="AB5">
-        <v>5.2590944147562577e-05</v>
+        <v>5.2590944147573203e-05</v>
       </c>
       <c r="AC5">
-        <v>-2.1056099340477884e-05</v>
+        <v>-2.1056099340469427e-05</v>
       </c>
       <c r="AD5">
-        <v>-5.3059972264982548e-06</v>
+        <v>-5.3059972264900691e-06</v>
       </c>
       <c r="AE5">
-        <v>-7.2812817573096904e-05</v>
+        <v>-7.2812817573086278e-05</v>
       </c>
       <c r="AF5">
-        <v>2.3800320149084932e-06</v>
+        <v>2.3800320149091234e-06</v>
       </c>
       <c r="AG5">
-        <v>0.00011273175229523135</v>
+        <v>0.00011273175229523005</v>
       </c>
       <c r="AH5">
-        <v>7.0103091909831813e-05</v>
+        <v>7.0103091909827909e-05</v>
       </c>
       <c r="AI5">
-        <v>-0.0020326920215607788</v>
+        <v>-0.0020326920215608581</v>
       </c>
     </row>
     <row r="6">
@@ -933,103 +933,103 @@
         <v>0.16250526351603703</v>
       </c>
       <c r="C6">
-        <v>-0.00010843423021864615</v>
+        <v>-0.00010843423021864604</v>
       </c>
       <c r="D6">
-        <v>0.0024417879512849943</v>
+        <v>0.0024417879512850195</v>
       </c>
       <c r="E6">
-        <v>0.0020642741812237952</v>
+        <v>0.0020642741812238186</v>
       </c>
       <c r="F6">
-        <v>0.0018612724534218567</v>
+        <v>0.0018612724534218779</v>
       </c>
       <c r="G6">
-        <v>0.057488003405249427</v>
+        <v>0.057488003405249455</v>
       </c>
       <c r="H6">
-        <v>0.0022753072320950917</v>
+        <v>0.0022753072320951104</v>
       </c>
       <c r="I6">
-        <v>0.001991292999147447</v>
+        <v>0.0019912929991474718</v>
       </c>
       <c r="J6">
-        <v>0.0021086397979223183</v>
+        <v>0.0021086397979223448</v>
       </c>
       <c r="K6">
-        <v>0.000499162153585417</v>
+        <v>0.0004991621535854222</v>
       </c>
       <c r="L6">
-        <v>0.00044981848966821586</v>
+        <v>0.00044981848966823651</v>
       </c>
       <c r="M6">
-        <v>0.00018633283427474867</v>
+        <v>0.0001863328342747504</v>
       </c>
       <c r="N6">
-        <v>0.00027573964584833103</v>
+        <v>0.00027573964584833504</v>
       </c>
       <c r="O6">
-        <v>0.00028512265825970701</v>
+        <v>0.00028512265825971189</v>
       </c>
       <c r="P6">
-        <v>-5.3984468993179338e-05</v>
+        <v>-5.398446899316687e-05</v>
       </c>
       <c r="Q6">
-        <v>6.9483088424569491e-05</v>
+        <v>6.9483088424646795e-05</v>
       </c>
       <c r="R6">
-        <v>-4.2746946247138073e-05</v>
+        <v>-4.2746946247127664e-05</v>
       </c>
       <c r="S6">
-        <v>0.0001053769319945768</v>
+        <v>0.00010537693199462651</v>
       </c>
       <c r="T6">
-        <v>0.00013915368209563547</v>
+        <v>0.00013915368209564504</v>
       </c>
       <c r="U6">
-        <v>0.00021119581025745267</v>
+        <v>0.00021119581025746525</v>
       </c>
       <c r="V6">
-        <v>0.00054653907747107444</v>
+        <v>0.00054653907747108572</v>
       </c>
       <c r="W6">
-        <v>0.0012059413454082234</v>
+        <v>0.0012059413454082583</v>
       </c>
       <c r="X6">
-        <v>-4.7557013707125948e-05</v>
+        <v>-4.7557013707125826e-05</v>
       </c>
       <c r="Y6">
-        <v>0.00012877618346038923</v>
+        <v>0.00012877618346038988</v>
       </c>
       <c r="Z6">
-        <v>0.00020423090026065174</v>
+        <v>0.00020423090026066562</v>
       </c>
       <c r="AA6">
-        <v>6.1444208924456853e-05</v>
+        <v>6.1444208924468779e-05</v>
       </c>
       <c r="AB6">
-        <v>0.0001231085885548299</v>
+        <v>0.00012310858855484356</v>
       </c>
       <c r="AC6">
-        <v>6.6073099431141315e-05</v>
+        <v>6.6073099431151507e-05</v>
       </c>
       <c r="AD6">
-        <v>2.2334027506154791e-05</v>
+        <v>2.233402750616547e-05</v>
       </c>
       <c r="AE6">
-        <v>-3.5116145501650625e-05</v>
+        <v>-3.5116145501637398e-05</v>
       </c>
       <c r="AF6">
-        <v>1.0130120580751479e-05</v>
+        <v>1.0130120580752258e-05</v>
       </c>
       <c r="AG6">
-        <v>-0.00013755789499182453</v>
+        <v>-0.00013755789499182583</v>
       </c>
       <c r="AH6">
-        <v>7.9445070357428687e-05</v>
+        <v>7.94450703574237e-05</v>
       </c>
       <c r="AI6">
-        <v>-0.0029729672163784247</v>
+        <v>-0.0029729672163785214</v>
       </c>
     </row>
     <row r="7">
@@ -1040,103 +1040,103 @@
         <v>-0.22492068207238639</v>
       </c>
       <c r="C7">
-        <v>-0.00010596516053969346</v>
+        <v>-0.00010596516053969373</v>
       </c>
       <c r="D7">
-        <v>0.0021134510801234059</v>
+        <v>0.0021134510801234241</v>
       </c>
       <c r="E7">
-        <v>0.0020977832497201653</v>
+        <v>0.0020977832497201827</v>
       </c>
       <c r="F7">
-        <v>0.0018492289694546063</v>
+        <v>0.0018492289694546213</v>
       </c>
       <c r="G7">
-        <v>0.0022753072320950917</v>
+        <v>0.0022753072320951104</v>
       </c>
       <c r="H7">
-        <v>0.0031113177501820512</v>
+        <v>0.0031113177501820698</v>
       </c>
       <c r="I7">
-        <v>0.0020203654061571332</v>
+        <v>0.0020203654061571588</v>
       </c>
       <c r="J7">
-        <v>0.0021083988136712008</v>
+        <v>0.0021083988136712272</v>
       </c>
       <c r="K7">
-        <v>0.00039531652231036374</v>
+        <v>0.00039531652231037046</v>
       </c>
       <c r="L7">
-        <v>0.00038087372306953724</v>
+        <v>0.00038087372306955822</v>
       </c>
       <c r="M7">
-        <v>0.00011825463761074928</v>
+        <v>0.00011825463761075037</v>
       </c>
       <c r="N7">
-        <v>0.00016660764644241399</v>
+        <v>0.000166607646442418</v>
       </c>
       <c r="O7">
-        <v>0.00010625670043667456</v>
+        <v>0.00010625670043667934</v>
       </c>
       <c r="P7">
-        <v>2.4952126135451978e-05</v>
+        <v>2.4952126135464555e-05</v>
       </c>
       <c r="Q7">
-        <v>1.6276286501519304e-06</v>
+        <v>1.6276286502292341e-06</v>
       </c>
       <c r="R7">
-        <v>-3.8034219591053182e-05</v>
+        <v>-3.8034219591042448e-05</v>
       </c>
       <c r="S7">
-        <v>3.104761253483148e-05</v>
+        <v>3.1047612534881083e-05</v>
       </c>
       <c r="T7">
-        <v>0.00013130352291067067</v>
+        <v>0.0001313035229106804</v>
       </c>
       <c r="U7">
-        <v>0.00014664378215088975</v>
+        <v>0.00014664378215090254</v>
       </c>
       <c r="V7">
-        <v>0.00051188472275484316</v>
+        <v>0.00051188472275485487</v>
       </c>
       <c r="W7">
-        <v>0.001063574258902799</v>
+        <v>0.0010635742589028341</v>
       </c>
       <c r="X7">
-        <v>-2.6566527801927502e-05</v>
+        <v>-2.6566527801927329e-05</v>
       </c>
       <c r="Y7">
-        <v>-1.8494888706545559e-05</v>
+        <v>-1.8494888706544908e-05</v>
       </c>
       <c r="Z7">
-        <v>0.00022190153581250639</v>
+        <v>0.00022190153581251983</v>
       </c>
       <c r="AA7">
-        <v>0.00014698745143087479</v>
+        <v>0.00014698745143088671</v>
       </c>
       <c r="AB7">
-        <v>0.00017526084095628117</v>
+        <v>0.00017526084095629484</v>
       </c>
       <c r="AC7">
-        <v>9.9242546054492892e-05</v>
+        <v>9.9242546054503084e-05</v>
       </c>
       <c r="AD7">
-        <v>0.00011251699848729887</v>
+        <v>0.00011251699848730922</v>
       </c>
       <c r="AE7">
-        <v>-6.6641415073845887e-06</v>
+        <v>-6.664141507371497e-06</v>
       </c>
       <c r="AF7">
-        <v>1.4003597577924943e-05</v>
+        <v>1.4003597577925736e-05</v>
       </c>
       <c r="AG7">
-        <v>-8.6778641401065969e-05</v>
+        <v>-8.677864140106727e-05</v>
       </c>
       <c r="AH7">
-        <v>6.0970632979302688e-05</v>
+        <v>6.0970632979297701e-05</v>
       </c>
       <c r="AI7">
-        <v>-0.0028559799727096713</v>
+        <v>-0.0028559799727097693</v>
       </c>
     </row>
     <row r="8">
@@ -1147,103 +1147,103 @@
         <v>-0.1529704486597758</v>
       </c>
       <c r="C8">
-        <v>0.00011732840928461018</v>
+        <v>0.00011732840928460902</v>
       </c>
       <c r="D8">
-        <v>0.0019828406336588871</v>
+        <v>0.0019828406336589123</v>
       </c>
       <c r="E8">
-        <v>0.0021085718188296109</v>
+        <v>0.0021085718188296331</v>
       </c>
       <c r="F8">
-        <v>0.001802882282930145</v>
+        <v>0.001802882282930165</v>
       </c>
       <c r="G8">
-        <v>0.001991292999147447</v>
+        <v>0.0019912929991474718</v>
       </c>
       <c r="H8">
-        <v>0.0020203654061571332</v>
+        <v>0.0020203654061571588</v>
       </c>
       <c r="I8">
-        <v>0.0023630518918623398</v>
+        <v>0.0023630518918623623</v>
       </c>
       <c r="J8">
-        <v>0.0021630154235348737</v>
+        <v>0.0021630154235348989</v>
       </c>
       <c r="K8">
-        <v>-9.6477412201960693e-05</v>
+        <v>-9.6477412201952453e-05</v>
       </c>
       <c r="L8">
-        <v>-6.2624319062020188e-05</v>
+        <v>-6.2624319062000184e-05</v>
       </c>
       <c r="M8">
-        <v>8.9623365210410788e-05</v>
+        <v>8.9623365210411872e-05</v>
       </c>
       <c r="N8">
-        <v>0.00012382017728425647</v>
+        <v>0.00012382017728426056</v>
       </c>
       <c r="O8">
-        <v>0.00012507577302552488</v>
+        <v>0.00012507577302552959</v>
       </c>
       <c r="P8">
-        <v>0.00012121079140615248</v>
+        <v>0.0001212107914061668</v>
       </c>
       <c r="Q8">
-        <v>-5.1614434372137608e-06</v>
+        <v>-5.1614434371389508e-06</v>
       </c>
       <c r="R8">
-        <v>-2.4039909615055483e-05</v>
+        <v>-2.4039909615042798e-05</v>
       </c>
       <c r="S8">
-        <v>-3.7246413668003554e-05</v>
+        <v>-3.7246413667954385e-05</v>
       </c>
       <c r="T8">
-        <v>9.1079901964059986e-05</v>
+        <v>9.1079901964069663e-05</v>
       </c>
       <c r="U8">
-        <v>0.00022175602752184205</v>
+        <v>0.00022175602752185462</v>
       </c>
       <c r="V8">
-        <v>0.0003513849927976253</v>
+        <v>0.00035138499279763918</v>
       </c>
       <c r="W8">
-        <v>0.000769543349896985</v>
+        <v>0.00076954334989701731</v>
       </c>
       <c r="X8">
-        <v>-3.6324449322708719e-05</v>
+        <v>-3.6324449322708611e-05</v>
       </c>
       <c r="Y8">
-        <v>-8.8974886706919552e-05</v>
+        <v>-8.8974886706918684e-05</v>
       </c>
       <c r="Z8">
-        <v>5.285445932202786e-05</v>
+        <v>5.2854459322041088e-05</v>
       </c>
       <c r="AA8">
-        <v>3.2123447875525299e-05</v>
+        <v>3.2123447875537442e-05</v>
       </c>
       <c r="AB8">
-        <v>5.362024703079349e-05</v>
+        <v>5.3620247030806501e-05</v>
       </c>
       <c r="AC8">
-        <v>-1.5459636173135441e-05</v>
+        <v>-1.54596361731259e-05</v>
       </c>
       <c r="AD8">
-        <v>3.2777159819301132e-05</v>
+        <v>3.2777159819310836e-05</v>
       </c>
       <c r="AE8">
-        <v>2.4805335383795338e-05</v>
+        <v>2.4805335383808186e-05</v>
       </c>
       <c r="AF8">
-        <v>2.8167527087327672e-06</v>
+        <v>2.8167527087335329e-06</v>
       </c>
       <c r="AG8">
-        <v>4.6806591355737746e-06</v>
+        <v>4.6806591355711726e-06</v>
       </c>
       <c r="AH8">
-        <v>3.7243755954839588e-05</v>
+        <v>3.7243755954834818e-05</v>
       </c>
       <c r="AI8">
-        <v>-0.0024133870012868893</v>
+        <v>-0.0024133870012869878</v>
       </c>
     </row>
     <row r="9">
@@ -1254,103 +1254,103 @@
         <v>-0.36025040732867963</v>
       </c>
       <c r="C9">
-        <v>0.00018803916794095022</v>
+        <v>0.00018803916794095035</v>
       </c>
       <c r="D9">
-        <v>0.0020871683533679178</v>
+        <v>0.0020871683533679438</v>
       </c>
       <c r="E9">
-        <v>0.0021090443932507389</v>
+        <v>0.0021090443932507631</v>
       </c>
       <c r="F9">
-        <v>0.0017667256002488313</v>
+        <v>0.0017667256002488528</v>
       </c>
       <c r="G9">
-        <v>0.0021086397979223183</v>
+        <v>0.0021086397979223448</v>
       </c>
       <c r="H9">
-        <v>0.0021083988136712008</v>
+        <v>0.0021083988136712272</v>
       </c>
       <c r="I9">
-        <v>0.0021630154235348737</v>
+        <v>0.0021630154235348989</v>
       </c>
       <c r="J9">
-        <v>0.0042791945053281084</v>
+        <v>0.0042791945053281336</v>
       </c>
       <c r="K9">
-        <v>0.00017945082029095587</v>
+        <v>0.00017945082029096368</v>
       </c>
       <c r="L9">
-        <v>4.5283576011172862e-05</v>
+        <v>4.528357601119441e-05</v>
       </c>
       <c r="M9">
-        <v>4.9604585912203271e-05</v>
+        <v>4.9604585912205439e-05</v>
       </c>
       <c r="N9">
-        <v>4.7138664410984951e-05</v>
+        <v>4.7138664410989125e-05</v>
       </c>
       <c r="O9">
-        <v>5.7869774781328644e-05</v>
+        <v>5.7869774781333665e-05</v>
       </c>
       <c r="P9">
-        <v>0.00020041402999989547</v>
+        <v>0.00020041402999990848</v>
       </c>
       <c r="Q9">
-        <v>6.3657106405295766e-05</v>
+        <v>6.3657106405375671e-05</v>
       </c>
       <c r="R9">
-        <v>-1.090278735531964e-05</v>
+        <v>-1.0902787355308852e-05</v>
       </c>
       <c r="S9">
-        <v>-6.0940037529625996e-05</v>
+        <v>-6.0940037529575038e-05</v>
       </c>
       <c r="T9">
-        <v>6.999213058396495e-05</v>
+        <v>6.999213058397506e-05</v>
       </c>
       <c r="U9">
-        <v>7.925130788153387e-05</v>
+        <v>7.9251307881547098e-05</v>
       </c>
       <c r="V9">
-        <v>0.0004394237064820612</v>
+        <v>0.00043942370648207335</v>
       </c>
       <c r="W9">
-        <v>0.00077552129634346251</v>
+        <v>0.00077552129634349829</v>
       </c>
       <c r="X9">
-        <v>-3.8749522387691831e-05</v>
+        <v>-3.8749522387691655e-05</v>
       </c>
       <c r="Y9">
-        <v>-2.3845104977733469e-05</v>
+        <v>-2.384510497773271e-05</v>
       </c>
       <c r="Z9">
-        <v>0.00014993704661024967</v>
+        <v>0.00014993704661026355</v>
       </c>
       <c r="AA9">
-        <v>0.00012300481935884349</v>
+        <v>0.00012300481935885563</v>
       </c>
       <c r="AB9">
-        <v>7.6264365752959753e-05</v>
+        <v>7.6264365752973414e-05</v>
       </c>
       <c r="AC9">
-        <v>7.7531048207134723e-05</v>
+        <v>7.7531048207145131e-05</v>
       </c>
       <c r="AD9">
-        <v>0.00016385404757253771</v>
+        <v>0.00016385404757254807</v>
       </c>
       <c r="AE9">
-        <v>1.1865457425506851e-05</v>
+        <v>1.1865457425520377e-05</v>
       </c>
       <c r="AF9">
-        <v>2.2537754202507757e-06</v>
+        <v>2.2537754202515888e-06</v>
       </c>
       <c r="AG9">
-        <v>0.00015386211925594567</v>
+        <v>0.00015386211925594393</v>
       </c>
       <c r="AH9">
-        <v>-2.3520691061540422e-05</v>
+        <v>-2.3520691061545192e-05</v>
       </c>
       <c r="AI9">
-        <v>-0.002582096142993707</v>
+        <v>-0.0025820961429938089</v>
       </c>
     </row>
     <row r="10">
@@ -1361,103 +1361,103 @@
         <v>0.15737459156980077</v>
       </c>
       <c r="C10">
-        <v>5.1197771764598007e-06</v>
+        <v>5.1197771764612237e-06</v>
       </c>
       <c r="D10">
-        <v>-2.0115308488022473e-05</v>
+        <v>-2.0115308488016619e-05</v>
       </c>
       <c r="E10">
-        <v>1.4118593225045939e-05</v>
+        <v>1.4118593225052661e-05</v>
       </c>
       <c r="F10">
-        <v>0.0001037959055400241</v>
+        <v>0.00010379590554003039</v>
       </c>
       <c r="G10">
-        <v>0.000499162153585417</v>
+        <v>0.0004991621535854222</v>
       </c>
       <c r="H10">
-        <v>0.00039531652231036374</v>
+        <v>0.00039531652231037046</v>
       </c>
       <c r="I10">
-        <v>-9.6477412201960693e-05</v>
+        <v>-9.6477412201952453e-05</v>
       </c>
       <c r="J10">
-        <v>0.00017945082029095587</v>
+        <v>0.00017945082029096368</v>
       </c>
       <c r="K10">
-        <v>0.0074102080942152846</v>
+        <v>0.0074102080942152811</v>
       </c>
       <c r="L10">
-        <v>0.0032290788500811763</v>
+        <v>0.0032290788500811923</v>
       </c>
       <c r="M10">
-        <v>-0.0040853893661426562</v>
+        <v>-0.0040853893661426553</v>
       </c>
       <c r="N10">
-        <v>7.6384446146617079e-05</v>
+        <v>7.6384446146619085e-05</v>
       </c>
       <c r="O10">
-        <v>0.00017008274704562862</v>
+        <v>0.00017008274704563168</v>
       </c>
       <c r="P10">
-        <v>0.00034860485841903114</v>
+        <v>0.00034860485841902724</v>
       </c>
       <c r="Q10">
-        <v>9.7647707584599822e-05</v>
+        <v>9.7647707584657718e-05</v>
       </c>
       <c r="R10">
-        <v>6.1269581888890234e-05</v>
+        <v>6.1269581888881127e-05</v>
       </c>
       <c r="S10">
-        <v>0.00016744100269595696</v>
+        <v>0.00016744100269598612</v>
       </c>
       <c r="T10">
-        <v>0.00063230654186255972</v>
+        <v>0.00063230654186256547</v>
       </c>
       <c r="U10">
-        <v>0.0032118980277105877</v>
+        <v>0.0032118980277105924</v>
       </c>
       <c r="V10">
-        <v>0.0036789130441664463</v>
+        <v>0.0036789130441664351</v>
       </c>
       <c r="W10">
-        <v>0.0039392190568509015</v>
+        <v>0.0039392190568509327</v>
       </c>
       <c r="X10">
-        <v>-0.00016679003225496483</v>
+        <v>-0.00016679003225496437</v>
       </c>
       <c r="Y10">
-        <v>3.7762544182087083e-05</v>
+        <v>3.7762544182086649e-05</v>
       </c>
       <c r="Z10">
-        <v>0.00018681899800963376</v>
+        <v>0.0001868189980096433</v>
       </c>
       <c r="AA10">
-        <v>0.00010292825587060895</v>
+        <v>0.00010292825587061589</v>
       </c>
       <c r="AB10">
-        <v>7.9016028483066278e-05</v>
+        <v>7.9016028483075602e-05</v>
       </c>
       <c r="AC10">
-        <v>0.0001535077105833311</v>
+        <v>0.00015350771058333999</v>
       </c>
       <c r="AD10">
-        <v>0.00035701943319050699</v>
+        <v>0.00035701943319051686</v>
       </c>
       <c r="AE10">
-        <v>0.0002187728275894843</v>
+        <v>0.00021877282758949387</v>
       </c>
       <c r="AF10">
-        <v>-3.2565980408890923e-07</v>
+        <v>-3.2565980408828582e-07</v>
       </c>
       <c r="AG10">
-        <v>0.00037063543131517608</v>
+        <v>0.00037063543131517695</v>
       </c>
       <c r="AH10">
-        <v>-9.4744370399680016e-05</v>
+        <v>-9.4744370399683486e-05</v>
       </c>
       <c r="AI10">
-        <v>-0.0040142065628919503</v>
+        <v>-0.0040142065628920171</v>
       </c>
     </row>
     <row r="11">
@@ -1468,103 +1468,103 @@
         <v>0.083971588068680172</v>
       </c>
       <c r="C11">
-        <v>-4.2400694082288633e-05</v>
+        <v>-4.2400694082287739e-05</v>
       </c>
       <c r="D11">
-        <v>0.0001862923207223158</v>
+        <v>0.0001862923207223358</v>
       </c>
       <c r="E11">
-        <v>-9.3260023870279937e-05</v>
+        <v>-9.3260023870260489e-05</v>
       </c>
       <c r="F11">
-        <v>9.6185840505532403e-05</v>
+        <v>9.6185840505550211e-05</v>
       </c>
       <c r="G11">
-        <v>0.00044981848966821586</v>
+        <v>0.00044981848966823651</v>
       </c>
       <c r="H11">
-        <v>0.00038087372306953724</v>
+        <v>0.00038087372306955822</v>
       </c>
       <c r="I11">
-        <v>-6.2624319062020188e-05</v>
+        <v>-6.2624319062000184e-05</v>
       </c>
       <c r="J11">
-        <v>4.5283576011172862e-05</v>
+        <v>4.528357601119441e-05</v>
       </c>
       <c r="K11">
-        <v>0.0032290788500811763</v>
+        <v>0.0032290788500811923</v>
       </c>
       <c r="L11">
-        <v>0.0031002153941946968</v>
+        <v>0.0031002153941947137</v>
       </c>
       <c r="M11">
-        <v>-0.00041434020189945052</v>
+        <v>-0.00041434020189944922</v>
       </c>
       <c r="N11">
-        <v>0.00015482852411966399</v>
+        <v>0.00015482852411966605</v>
       </c>
       <c r="O11">
-        <v>8.2149596255874971e-05</v>
+        <v>8.21495962558784e-05</v>
       </c>
       <c r="P11">
-        <v>0.00030185717532583457</v>
+        <v>0.0003018571753258311</v>
       </c>
       <c r="Q11">
-        <v>0.00017023512700279297</v>
+        <v>0.00017023512700285585</v>
       </c>
       <c r="R11">
-        <v>0.00028235702247508392</v>
+        <v>0.00028235702247507617</v>
       </c>
       <c r="S11">
-        <v>0.00047732123564773365</v>
+        <v>0.00047732123564776666</v>
       </c>
       <c r="T11">
-        <v>0.00047289903568890847</v>
+        <v>0.00047289903568891465</v>
       </c>
       <c r="U11">
-        <v>0.0026454966364136681</v>
+        <v>0.002645496636413675</v>
       </c>
       <c r="V11">
-        <v>0.0030849932598246382</v>
+        <v>0.0030849932598246296</v>
       </c>
       <c r="W11">
-        <v>0.0033259568499667243</v>
+        <v>0.003325956849966759</v>
       </c>
       <c r="X11">
-        <v>-0.0001492195673697877</v>
+        <v>-0.00014921956736978716</v>
       </c>
       <c r="Y11">
-        <v>4.2739638244125274e-05</v>
+        <v>4.2739638244124894e-05</v>
       </c>
       <c r="Z11">
-        <v>4.4432803402145657e-05</v>
+        <v>4.4432803402155632e-05</v>
       </c>
       <c r="AA11">
-        <v>-5.0739540888786183e-05</v>
+        <v>-5.0739540888778811e-05</v>
       </c>
       <c r="AB11">
-        <v>-2.6403228015850705e-05</v>
+        <v>-2.6403228015840947e-05</v>
       </c>
       <c r="AC11">
-        <v>2.9783468960469656e-05</v>
+        <v>2.9783468960480498e-05</v>
       </c>
       <c r="AD11">
-        <v>0.00011865440852693141</v>
+        <v>0.00011865440852694214</v>
       </c>
       <c r="AE11">
-        <v>-5.003866963365614e-05</v>
+        <v>-5.0038669633645488e-05</v>
       </c>
       <c r="AF11">
-        <v>1.0516857342269178e-05</v>
+        <v>1.0516857342269856e-05</v>
       </c>
       <c r="AG11">
         <v>5.5955232594965317e-05</v>
       </c>
       <c r="AH11">
-        <v>-2.7635679663996337e-05</v>
+        <v>-2.7635679664000023e-05</v>
       </c>
       <c r="AI11">
-        <v>-0.0036131444182356887</v>
+        <v>-0.0036131444182357572</v>
       </c>
     </row>
     <row r="12">
@@ -1575,103 +1575,103 @@
         <v>-0.05101015186102266</v>
       </c>
       <c r="C12">
-        <v>-6.0906119824910346e-05</v>
+        <v>-6.0906119824910264e-05</v>
       </c>
       <c r="D12">
-        <v>0.00027309987750996157</v>
+        <v>0.00027309987750996309</v>
       </c>
       <c r="E12">
-        <v>0.00011537275032906199</v>
+        <v>0.00011537275032906373</v>
       </c>
       <c r="F12">
-        <v>8.1680466308312917e-05</v>
+        <v>8.1680466308314218e-05</v>
       </c>
       <c r="G12">
-        <v>0.00018633283427474867</v>
+        <v>0.0001863328342747504</v>
       </c>
       <c r="H12">
-        <v>0.00011825463761074928</v>
+        <v>0.00011825463761075037</v>
       </c>
       <c r="I12">
-        <v>8.9623365210410788e-05</v>
+        <v>8.9623365210411872e-05</v>
       </c>
       <c r="J12">
-        <v>4.9604585912203271e-05</v>
+        <v>4.9604585912205439e-05</v>
       </c>
       <c r="K12">
-        <v>-0.0040853893661426562</v>
+        <v>-0.0040853893661426553</v>
       </c>
       <c r="L12">
-        <v>-0.00041434020189945052</v>
+        <v>-0.00041434020189944922</v>
       </c>
       <c r="M12">
         <v>0.0056550742588793567</v>
       </c>
       <c r="N12">
-        <v>0.00053972298045773537</v>
+        <v>0.00053972298045773558</v>
       </c>
       <c r="O12">
-        <v>0.00041312332789258054</v>
+        <v>0.00041312332789258098</v>
       </c>
       <c r="P12">
-        <v>0.00015702916722206293</v>
+        <v>0.0001570291672220638</v>
       </c>
       <c r="Q12">
-        <v>8.1640007173089296e-05</v>
+        <v>8.1640007173097549e-05</v>
       </c>
       <c r="R12">
-        <v>8.659241108307745e-05</v>
+        <v>8.659241108307806e-05</v>
       </c>
       <c r="S12">
-        <v>7.2625568124505723e-05</v>
+        <v>7.2625568124509883e-05</v>
       </c>
       <c r="T12">
-        <v>-0.00021872529679949171</v>
+        <v>-0.00021872529679949068</v>
       </c>
       <c r="U12">
-        <v>-0.00055939481065233362</v>
+        <v>-0.00055939481065233254</v>
       </c>
       <c r="V12">
-        <v>-0.00045654085313738161</v>
+        <v>-0.00045654085313738102</v>
       </c>
       <c r="W12">
-        <v>-0.00033281241228975955</v>
+        <v>-0.00033281241228975544</v>
       </c>
       <c r="X12">
-        <v>1.3508018690001934e-05</v>
+        <v>1.3508018690001983e-05</v>
       </c>
       <c r="Y12">
-        <v>3.3516023083526297e-06</v>
+        <v>3.3516023083527584e-06</v>
       </c>
       <c r="Z12">
-        <v>5.3753552470530829e-06</v>
+        <v>5.3753552470534624e-06</v>
       </c>
       <c r="AA12">
-        <v>-4.7040608925575636e-05</v>
+        <v>-4.7040608925574498e-05</v>
       </c>
       <c r="AB12">
-        <v>2.4527032191439961e-05</v>
+        <v>2.4527032191441208e-05</v>
       </c>
       <c r="AC12">
-        <v>-2.7358458102672961e-05</v>
+        <v>-2.7358458102671876e-05</v>
       </c>
       <c r="AD12">
-        <v>-7.4634030212139476e-05</v>
+        <v>-7.4634030212138337e-05</v>
       </c>
       <c r="AE12">
-        <v>-0.00015014202061696563</v>
+        <v>-0.00015014202061696452</v>
       </c>
       <c r="AF12">
-        <v>1.4859872921433072e-05</v>
+        <v>1.4859872921433194e-05</v>
       </c>
       <c r="AG12">
-        <v>-0.00030833222323535297</v>
+        <v>-0.0003083322232353533</v>
       </c>
       <c r="AH12">
-        <v>-4.2100416755658121e-05</v>
+        <v>-4.2100416755658744e-05</v>
       </c>
       <c r="AI12">
-        <v>-0.00015965131485163437</v>
+        <v>-0.00015965131485163692</v>
       </c>
     </row>
     <row r="13">
@@ -1682,103 +1682,103 @@
         <v>-0.080449105696533005</v>
       </c>
       <c r="C13">
-        <v>-3.361322185230121e-05</v>
+        <v>-3.3613221852301075e-05</v>
       </c>
       <c r="D13">
-        <v>3.415495757352156e-05</v>
+        <v>3.4154957573525626e-05</v>
       </c>
       <c r="E13">
-        <v>0.00013157663846053444</v>
+        <v>0.00013157663846053829</v>
       </c>
       <c r="F13">
-        <v>0.00012419560983464682</v>
+        <v>0.00012419560983465032</v>
       </c>
       <c r="G13">
-        <v>0.00027573964584833103</v>
+        <v>0.00027573964584833504</v>
       </c>
       <c r="H13">
-        <v>0.00016660764644241399</v>
+        <v>0.000166607646442418</v>
       </c>
       <c r="I13">
-        <v>0.00012382017728425647</v>
+        <v>0.00012382017728426056</v>
       </c>
       <c r="J13">
-        <v>4.7138664410984951e-05</v>
+        <v>4.7138664410989125e-05</v>
       </c>
       <c r="K13">
-        <v>7.6384446146617079e-05</v>
+        <v>7.6384446146619085e-05</v>
       </c>
       <c r="L13">
-        <v>0.00015482852411966399</v>
+        <v>0.00015482852411966605</v>
       </c>
       <c r="M13">
-        <v>0.00053972298045773537</v>
+        <v>0.00053972298045773558</v>
       </c>
       <c r="N13">
-        <v>0.00085714983948552209</v>
+        <v>0.00085714983948552241</v>
       </c>
       <c r="O13">
-        <v>0.00042212863405599837</v>
+        <v>0.00042212863405599924</v>
       </c>
       <c r="P13">
-        <v>0.00023414186729393713</v>
+        <v>0.0002341418672939381</v>
       </c>
       <c r="Q13">
-        <v>3.9947432961129814e-05</v>
+        <v>3.994743296114258e-05</v>
       </c>
       <c r="R13">
-        <v>-1.9673944736484721e-05</v>
+        <v>-1.967394473648407e-05</v>
       </c>
       <c r="S13">
-        <v>4.0788415143500092e-05</v>
+        <v>4.0788415143506556e-05</v>
       </c>
       <c r="T13">
-        <v>-2.4394818592365961e-05</v>
+        <v>-2.4394818592364416e-05</v>
       </c>
       <c r="U13">
-        <v>0.00014571898141819267</v>
+        <v>0.00014571898141819425</v>
       </c>
       <c r="V13">
-        <v>0.00024170927075665868</v>
+        <v>0.00024170927075665923</v>
       </c>
       <c r="W13">
-        <v>0.00043867877034087726</v>
+        <v>0.00043867877034088393</v>
       </c>
       <c r="X13">
-        <v>-8.9450452029444165e-06</v>
+        <v>-8.94504520294432e-06</v>
       </c>
       <c r="Y13">
-        <v>2.5349901746122248e-06</v>
+        <v>2.5349901746123875e-06</v>
       </c>
       <c r="Z13">
-        <v>3.176840152891992e-05</v>
+        <v>3.176840152892095e-05</v>
       </c>
       <c r="AA13">
-        <v>1.4427976619051325e-05</v>
+        <v>1.4427976619053114e-05</v>
       </c>
       <c r="AB13">
-        <v>4.8685890455250794e-06</v>
+        <v>4.8685890455269767e-06</v>
       </c>
       <c r="AC13">
-        <v>1.6549667470975769e-05</v>
+        <v>1.6549667470977449e-05</v>
       </c>
       <c r="AD13">
-        <v>1.0462524298719981e-05</v>
+        <v>1.0462524298721825e-05</v>
       </c>
       <c r="AE13">
-        <v>-2.3821879086441338e-05</v>
+        <v>-2.3821879086439562e-05</v>
       </c>
       <c r="AF13">
-        <v>5.616813985184142e-06</v>
+        <v>5.6168139851843385e-06</v>
       </c>
       <c r="AG13">
-        <v>-9.8069252881486258e-05</v>
+        <v>-9.8069252881486746e-05</v>
       </c>
       <c r="AH13">
-        <v>-3.6525377833204319e-05</v>
+        <v>-3.6525377833205295e-05</v>
       </c>
       <c r="AI13">
-        <v>-0.00082028153442178608</v>
+        <v>-0.00082028153442179996</v>
       </c>
     </row>
     <row r="14">
@@ -1789,103 +1789,103 @@
         <v>-0.028886584725227402</v>
       </c>
       <c r="C14">
-        <v>-4.8211227158035332e-05</v>
+        <v>-4.8211227158035095e-05</v>
       </c>
       <c r="D14">
-        <v>0.00017304750110305124</v>
+        <v>0.00017304750110305598</v>
       </c>
       <c r="E14">
-        <v>9.2101658019669966e-05</v>
+        <v>9.2101658019674547e-05</v>
       </c>
       <c r="F14">
-        <v>0.00011222399271491033</v>
+        <v>0.00011222399271491425</v>
       </c>
       <c r="G14">
-        <v>0.00028512265825970701</v>
+        <v>0.00028512265825971189</v>
       </c>
       <c r="H14">
-        <v>0.00010625670043667456</v>
+        <v>0.00010625670043667934</v>
       </c>
       <c r="I14">
-        <v>0.00012507577302552488</v>
+        <v>0.00012507577302552959</v>
       </c>
       <c r="J14">
-        <v>5.7869774781328644e-05</v>
+        <v>5.7869774781333665e-05</v>
       </c>
       <c r="K14">
-        <v>0.00017008274704562862</v>
+        <v>0.00017008274704563168</v>
       </c>
       <c r="L14">
-        <v>8.2149596255874971e-05</v>
+        <v>8.21495962558784e-05</v>
       </c>
       <c r="M14">
-        <v>0.00041312332789258054</v>
+        <v>0.00041312332789258098</v>
       </c>
       <c r="N14">
-        <v>0.00042212863405599837</v>
+        <v>0.00042212863405599924</v>
       </c>
       <c r="O14">
-        <v>0.00078169302244828506</v>
+        <v>0.00078169302244828637</v>
       </c>
       <c r="P14">
-        <v>3.2044993063426854e-05</v>
+        <v>3.2044993063428642e-05</v>
       </c>
       <c r="Q14">
-        <v>0.00012321554516546714</v>
+        <v>0.00012321554516548573</v>
       </c>
       <c r="R14">
-        <v>0.00021635474993374584</v>
+        <v>0.0002163547499337467</v>
       </c>
       <c r="S14">
-        <v>0.00031014633916723653</v>
+        <v>0.00031014633916724515</v>
       </c>
       <c r="T14">
-        <v>2.4679496354268625e-05</v>
+        <v>2.4679496354270889e-05</v>
       </c>
       <c r="U14">
-        <v>0.00018782629432656083</v>
+        <v>0.00018782629432656311</v>
       </c>
       <c r="V14">
-        <v>0.00029188576739535427</v>
+        <v>0.00029188576739535514</v>
       </c>
       <c r="W14">
-        <v>0.00050573604431693045</v>
+        <v>0.00050573604431693945</v>
       </c>
       <c r="X14">
-        <v>-1.0285577321125531e-05</v>
+        <v>-1.0285577321125419e-05</v>
       </c>
       <c r="Y14">
-        <v>1.0451598659236535e-05</v>
+        <v>1.0451598659236752e-05</v>
       </c>
       <c r="Z14">
-        <v>7.8399976348818355e-05</v>
+        <v>7.8399976348820632e-05</v>
       </c>
       <c r="AA14">
-        <v>8.0597869771119454e-05</v>
+        <v>8.0597869771121947e-05</v>
       </c>
       <c r="AB14">
-        <v>0.00010319506017073969</v>
+        <v>0.0001031950601707424</v>
       </c>
       <c r="AC14">
-        <v>1.7201678399737103e-05</v>
+        <v>1.7201678399739488e-05</v>
       </c>
       <c r="AD14">
-        <v>6.7471731706362253e-05</v>
+        <v>6.7471731706364855e-05</v>
       </c>
       <c r="AE14">
-        <v>1.4188838300472849e-05</v>
+        <v>1.4188838300475437e-05</v>
       </c>
       <c r="AF14">
-        <v>9.5812939870465262e-06</v>
+        <v>9.5812939870467515e-06</v>
       </c>
       <c r="AG14">
-        <v>-8.9809283282528017e-05</v>
+        <v>-8.9809283282528667e-05</v>
       </c>
       <c r="AH14">
-        <v>-7.0967816654567714e-05</v>
+        <v>-7.0967816654568961e-05</v>
       </c>
       <c r="AI14">
-        <v>-0.0011770786664807337</v>
+        <v>-0.0011770786664807545</v>
       </c>
     </row>
     <row r="15">
@@ -1896,103 +1896,103 @@
         <v>-0.11485641027320445</v>
       </c>
       <c r="C15">
-        <v>0.00015964187899656531</v>
+        <v>0.00015964187899656515</v>
       </c>
       <c r="D15">
-        <v>0.00024098226622748672</v>
+        <v>0.00024098226622749843</v>
       </c>
       <c r="E15">
-        <v>0.00025685583857601392</v>
+        <v>0.00025685583857602715</v>
       </c>
       <c r="F15">
-        <v>2.6036874602798177e-05</v>
+        <v>2.6036874602808802e-05</v>
       </c>
       <c r="G15">
-        <v>-5.3984468993179338e-05</v>
+        <v>-5.398446899316687e-05</v>
       </c>
       <c r="H15">
-        <v>2.4952126135451978e-05</v>
+        <v>2.4952126135464555e-05</v>
       </c>
       <c r="I15">
-        <v>0.00012121079140615248</v>
+        <v>0.0001212107914061668</v>
       </c>
       <c r="J15">
-        <v>0.00020041402999989547</v>
+        <v>0.00020041402999990848</v>
       </c>
       <c r="K15">
-        <v>0.00034860485841903114</v>
+        <v>0.00034860485841902724</v>
       </c>
       <c r="L15">
-        <v>0.00030185717532583457</v>
+        <v>0.0003018571753258311</v>
       </c>
       <c r="M15">
-        <v>0.00015702916722206293</v>
+        <v>0.0001570291672220638</v>
       </c>
       <c r="N15">
-        <v>0.00023414186729393713</v>
+        <v>0.0002341418672939381</v>
       </c>
       <c r="O15">
-        <v>3.2044993063426854e-05</v>
+        <v>3.2044993063428642e-05</v>
       </c>
       <c r="P15">
-        <v>0.009426341629225508</v>
+        <v>0.0094263416292255289</v>
       </c>
       <c r="Q15">
-        <v>0.0068137726272689426</v>
+        <v>0.0068137726272691195</v>
       </c>
       <c r="R15">
-        <v>0.0067577625961099744</v>
+        <v>0.0067577625961099935</v>
       </c>
       <c r="S15">
-        <v>0.0067408136400644997</v>
+        <v>0.0067408136400645769</v>
       </c>
       <c r="T15">
-        <v>-0.00011777917643881022</v>
+        <v>-0.00011777917643879086</v>
       </c>
       <c r="U15">
-        <v>0.00038688893363880315</v>
+        <v>0.00038688893363882744</v>
       </c>
       <c r="V15">
-        <v>0.00055400873771308933</v>
+        <v>0.00055400873771309887</v>
       </c>
       <c r="W15">
-        <v>0.00046371833807942004</v>
+        <v>0.00046371833807950721</v>
       </c>
       <c r="X15">
-        <v>-2.9039404761879379e-05</v>
+        <v>-2.9039404761877563e-05</v>
       </c>
       <c r="Y15">
-        <v>-0.00011733515753141401</v>
+        <v>-0.00011733515753141271</v>
       </c>
       <c r="Z15">
-        <v>0.00011420262847560651</v>
+        <v>0.00011420262847562559</v>
       </c>
       <c r="AA15">
-        <v>0.00016597672273013959</v>
+        <v>0.00016597672273016388</v>
       </c>
       <c r="AB15">
-        <v>0.00016024217855355183</v>
+        <v>0.00016024217855357525</v>
       </c>
       <c r="AC15">
-        <v>0.00011097867444821892</v>
+        <v>0.00011097867444824234</v>
       </c>
       <c r="AD15">
-        <v>0.00021100525375209183</v>
+        <v>0.00021100525375211568</v>
       </c>
       <c r="AE15">
-        <v>0.00039010103324478698</v>
+        <v>0.0003901010332448111</v>
       </c>
       <c r="AF15">
-        <v>5.7254640730687004e-06</v>
+        <v>5.7254640730701912e-06</v>
       </c>
       <c r="AG15">
-        <v>1.2088203191898579e-05</v>
+        <v>1.2088203191894242e-05</v>
       </c>
       <c r="AH15">
-        <v>-4.9005125978268584e-05</v>
+        <v>-4.9005125978278993e-05</v>
       </c>
       <c r="AI15">
-        <v>-0.007646923409067169</v>
+        <v>-0.0076469234090673632</v>
       </c>
     </row>
     <row r="16">
@@ -2003,103 +2003,103 @@
         <v>-0.099438391666721845</v>
       </c>
       <c r="C16">
-        <v>-2.9367506558327801e-05</v>
+        <v>-2.9367506558323816e-05</v>
       </c>
       <c r="D16">
-        <v>0.0002049088881617481</v>
+        <v>0.00020490888816182367</v>
       </c>
       <c r="E16">
-        <v>7.6911989027215739e-05</v>
+        <v>7.6911989027287839e-05</v>
       </c>
       <c r="F16">
-        <v>3.0606587825475549e-05</v>
+        <v>3.0606587825537783e-05</v>
       </c>
       <c r="G16">
-        <v>6.9483088424569491e-05</v>
+        <v>6.9483088424646795e-05</v>
       </c>
       <c r="H16">
-        <v>1.6276286501519304e-06</v>
+        <v>1.6276286502292341e-06</v>
       </c>
       <c r="I16">
-        <v>-5.1614434372137608e-06</v>
+        <v>-5.1614434371389508e-06</v>
       </c>
       <c r="J16">
-        <v>6.3657106405295766e-05</v>
+        <v>6.3657106405375671e-05</v>
       </c>
       <c r="K16">
-        <v>9.7647707584599822e-05</v>
+        <v>9.7647707584657718e-05</v>
       </c>
       <c r="L16">
-        <v>0.00017023512700279297</v>
+        <v>0.00017023512700285585</v>
       </c>
       <c r="M16">
-        <v>8.1640007173089296e-05</v>
+        <v>8.1640007173097549e-05</v>
       </c>
       <c r="N16">
-        <v>3.9947432961129814e-05</v>
+        <v>3.994743296114258e-05</v>
       </c>
       <c r="O16">
-        <v>0.00012321554516546714</v>
+        <v>0.00012321554516548573</v>
       </c>
       <c r="P16">
-        <v>0.0068137726272689426</v>
+        <v>0.0068137726272691195</v>
       </c>
       <c r="Q16">
-        <v>0.0073181904543887701</v>
+        <v>0.0073181904543889479</v>
       </c>
       <c r="R16">
-        <v>0.0069913547073796947</v>
+        <v>0.0069913547073797138</v>
       </c>
       <c r="S16">
-        <v>0.0070188449262131893</v>
+        <v>0.0070188449262132691</v>
       </c>
       <c r="T16">
-        <v>-0.00019017400239543304</v>
+        <v>-0.00019017400239541336</v>
       </c>
       <c r="U16">
-        <v>-2.4202738745484134e-07</v>
+        <v>-2.4202738742925417e-07</v>
       </c>
       <c r="V16">
-        <v>-2.6207257167606968e-05</v>
+        <v>-2.6207257167597427e-05</v>
       </c>
       <c r="W16">
-        <v>1.6812808064698651e-05</v>
+        <v>1.6812808064787556e-05</v>
       </c>
       <c r="X16">
-        <v>-1.5446679067544567e-05</v>
+        <v>-1.5446679067542744e-05</v>
       </c>
       <c r="Y16">
-        <v>-2.0611295039211402e-05</v>
+        <v>-2.0611295039210317e-05</v>
       </c>
       <c r="Z16">
-        <v>0.00039977578339571874</v>
+        <v>0.00039977578339573782</v>
       </c>
       <c r="AA16">
-        <v>0.00039619269341183844</v>
+        <v>0.00039619269341186359</v>
       </c>
       <c r="AB16">
-        <v>0.00039999263156205271</v>
+        <v>0.00039999263156207613</v>
       </c>
       <c r="AC16">
-        <v>0.00032778991844844511</v>
+        <v>0.00032778991844847026</v>
       </c>
       <c r="AD16">
-        <v>0.00040526383753041113</v>
+        <v>0.00040526383753043585</v>
       </c>
       <c r="AE16">
-        <v>0.00037619705005900988</v>
+        <v>0.00037619705005903449</v>
       </c>
       <c r="AF16">
-        <v>-2.857098044788532e-07</v>
+        <v>-2.8570980447728111e-07</v>
       </c>
       <c r="AG16">
-        <v>4.3779515320177889e-05</v>
+        <v>4.3779515320172685e-05</v>
       </c>
       <c r="AH16">
-        <v>2.3744716712641081e-05</v>
+        <v>2.3744716712629371e-05</v>
       </c>
       <c r="AI16">
-        <v>-0.0074153616530795467</v>
+        <v>-0.0074153616530797445</v>
       </c>
     </row>
     <row r="17">
@@ -2110,103 +2110,103 @@
         <v>-0.083042836433586745</v>
       </c>
       <c r="C17">
-        <v>-5.3783345333062307e-05</v>
+        <v>-5.3783345333062239e-05</v>
       </c>
       <c r="D17">
-        <v>0.00013961429365073885</v>
+        <v>0.00013961429365074959</v>
       </c>
       <c r="E17">
-        <v>5.8410909162380639e-05</v>
+        <v>5.8410909162392619e-05</v>
       </c>
       <c r="F17">
-        <v>-5.2813169843047366e-06</v>
+        <v>-5.2813169842945993e-06</v>
       </c>
       <c r="G17">
-        <v>-4.2746946247138073e-05</v>
+        <v>-4.2746946247127664e-05</v>
       </c>
       <c r="H17">
-        <v>-3.8034219591053182e-05</v>
+        <v>-3.8034219591042448e-05</v>
       </c>
       <c r="I17">
-        <v>-2.4039909615055483e-05</v>
+        <v>-2.4039909615042798e-05</v>
       </c>
       <c r="J17">
-        <v>-1.090278735531964e-05</v>
+        <v>-1.0902787355308852e-05</v>
       </c>
       <c r="K17">
-        <v>6.1269581888890234e-05</v>
+        <v>6.1269581888881127e-05</v>
       </c>
       <c r="L17">
-        <v>0.00028235702247508392</v>
+        <v>0.00028235702247507617</v>
       </c>
       <c r="M17">
-        <v>8.659241108307745e-05</v>
+        <v>8.659241108307806e-05</v>
       </c>
       <c r="N17">
-        <v>-1.9673944736484721e-05</v>
+        <v>-1.967394473648407e-05</v>
       </c>
       <c r="O17">
-        <v>0.00021635474993374584</v>
+        <v>0.0002163547499337467</v>
       </c>
       <c r="P17">
-        <v>0.0067577625961099744</v>
+        <v>0.0067577625961099935</v>
       </c>
       <c r="Q17">
-        <v>0.0069913547073796947</v>
+        <v>0.0069913547073797138</v>
       </c>
       <c r="R17">
-        <v>0.0072937728143594328</v>
+        <v>0.0072937728143594536</v>
       </c>
       <c r="S17">
-        <v>0.0071502877158113286</v>
+        <v>0.0071502877158114101</v>
       </c>
       <c r="T17">
-        <v>-0.00015611331133342095</v>
+        <v>-0.00015611331133340083</v>
       </c>
       <c r="U17">
-        <v>6.7493561899841393e-05</v>
+        <v>6.7493561899867414e-05</v>
       </c>
       <c r="V17">
-        <v>-1.1335263924642028e-05</v>
+        <v>-1.1335263924633354e-05</v>
       </c>
       <c r="W17">
-        <v>5.8702360032054837e-05</v>
+        <v>5.870236003214591e-05</v>
       </c>
       <c r="X17">
-        <v>-1.4914311524460619e-05</v>
+        <v>-1.4914311524458736e-05</v>
       </c>
       <c r="Y17">
-        <v>-2.791809035572186e-05</v>
+        <v>-2.7918090355720342e-05</v>
       </c>
       <c r="Z17">
-        <v>0.00042834881384021077</v>
+        <v>0.00042834881384023072</v>
       </c>
       <c r="AA17">
-        <v>0.00038964786848787094</v>
+        <v>0.00038964786848789609</v>
       </c>
       <c r="AB17">
-        <v>0.00039390262233660652</v>
+        <v>0.00039390262233663341</v>
       </c>
       <c r="AC17">
-        <v>0.00031836766960773727</v>
+        <v>0.00031836766960776329</v>
       </c>
       <c r="AD17">
-        <v>0.00039693324408751564</v>
+        <v>0.00039693324408754101</v>
       </c>
       <c r="AE17">
-        <v>0.00041366543595435884</v>
+        <v>0.0004136654359543841</v>
       </c>
       <c r="AF17">
-        <v>3.6208117601797146e-06</v>
+        <v>3.6208117601813138e-06</v>
       </c>
       <c r="AG17">
-        <v>4.5946337358625244e-05</v>
+        <v>4.594633735862351e-05</v>
       </c>
       <c r="AH17">
-        <v>2.3263439245871376e-05</v>
+        <v>2.3263439245859233e-05</v>
       </c>
       <c r="AI17">
-        <v>-0.0076541926183776501</v>
+        <v>-0.007654192618377853</v>
       </c>
     </row>
     <row r="18">
@@ -2217,103 +2217,103 @@
         <v>-0.13606630682082815</v>
       </c>
       <c r="C18">
-        <v>-0.00011313088460214999</v>
+        <v>-0.00011313088460214739</v>
       </c>
       <c r="D18">
-        <v>0.00035347518107974138</v>
+        <v>0.00035347518107978909</v>
       </c>
       <c r="E18">
-        <v>0.00011723908016807649</v>
+        <v>0.00011723908016812289</v>
       </c>
       <c r="F18">
-        <v>2.2049062175248733e-05</v>
+        <v>2.2049062175289933e-05</v>
       </c>
       <c r="G18">
-        <v>0.0001053769319945768</v>
+        <v>0.00010537693199462651</v>
       </c>
       <c r="H18">
-        <v>3.104761253483148e-05</v>
+        <v>3.1047612534881083e-05</v>
       </c>
       <c r="I18">
-        <v>-3.7246413668003554e-05</v>
+        <v>-3.7246413667954385e-05</v>
       </c>
       <c r="J18">
-        <v>-6.0940037529625996e-05</v>
+        <v>-6.0940037529575038e-05</v>
       </c>
       <c r="K18">
-        <v>0.00016744100269595696</v>
+        <v>0.00016744100269598612</v>
       </c>
       <c r="L18">
-        <v>0.00047732123564773365</v>
+        <v>0.00047732123564776666</v>
       </c>
       <c r="M18">
-        <v>7.2625568124505723e-05</v>
+        <v>7.2625568124509883e-05</v>
       </c>
       <c r="N18">
-        <v>4.0788415143500092e-05</v>
+        <v>4.0788415143506556e-05</v>
       </c>
       <c r="O18">
-        <v>0.00031014633916723653</v>
+        <v>0.00031014633916724515</v>
       </c>
       <c r="P18">
-        <v>0.0067408136400644997</v>
+        <v>0.0067408136400645769</v>
       </c>
       <c r="Q18">
-        <v>0.0070188449262131893</v>
+        <v>0.0070188449262132691</v>
       </c>
       <c r="R18">
-        <v>0.0071502877158113286</v>
+        <v>0.0071502877158114101</v>
       </c>
       <c r="S18">
-        <v>0.0077670221172790868</v>
+        <v>0.0077670221172791675</v>
       </c>
       <c r="T18">
-        <v>-0.00021038681129576778</v>
+        <v>-0.00021038681129574739</v>
       </c>
       <c r="U18">
-        <v>0.00017642226562673922</v>
+        <v>0.0001764222656267648</v>
       </c>
       <c r="V18">
-        <v>0.00013642230501540332</v>
+        <v>0.00013642230501541286</v>
       </c>
       <c r="W18">
-        <v>0.00025997622043381517</v>
+        <v>0.00025997622043390668</v>
       </c>
       <c r="X18">
-        <v>-1.2964826891340041e-05</v>
+        <v>-1.2964826891338069e-05</v>
       </c>
       <c r="Y18">
-        <v>1.2286128425974523e-06</v>
+        <v>1.2286128425987534e-06</v>
       </c>
       <c r="Z18">
-        <v>0.00050815612522661473</v>
+        <v>0.00050815612522663554</v>
       </c>
       <c r="AA18">
-        <v>0.00043808842808900489</v>
+        <v>0.00043808842808903178</v>
       </c>
       <c r="AB18">
-        <v>0.00045272675287770861</v>
+        <v>0.00045272675287773376</v>
       </c>
       <c r="AC18">
-        <v>0.00038264462745451165</v>
+        <v>0.00038264462745453767</v>
       </c>
       <c r="AD18">
-        <v>0.00049446962267037727</v>
+        <v>0.00049446962267040286</v>
       </c>
       <c r="AE18">
-        <v>0.00032125317013082764</v>
+        <v>0.0003212531701308536</v>
       </c>
       <c r="AF18">
-        <v>6.4351374456237591e-06</v>
+        <v>6.4351374456253854e-06</v>
       </c>
       <c r="AG18">
-        <v>4.3708144531398943e-05</v>
+        <v>4.3708144531393739e-05</v>
       </c>
       <c r="AH18">
-        <v>7.8244783439976838e-05</v>
+        <v>7.8244783439965129e-05</v>
       </c>
       <c r="AI18">
-        <v>-0.0080109756220309476</v>
+        <v>-0.0080109756220311541</v>
       </c>
     </row>
     <row r="19">
@@ -2324,103 +2324,103 @@
         <v>0.19475512354932451</v>
       </c>
       <c r="C19">
-        <v>3.3585706080962048e-07</v>
+        <v>3.3585706081016427e-07</v>
       </c>
       <c r="D19">
-        <v>-1.9174180004394734e-05</v>
+        <v>-1.9174180004385085e-05</v>
       </c>
       <c r="E19">
-        <v>7.8675240484065185e-05</v>
+        <v>7.8675240484074415e-05</v>
       </c>
       <c r="F19">
-        <v>3.3185996693455404e-05</v>
+        <v>3.3185996693463644e-05</v>
       </c>
       <c r="G19">
-        <v>0.00013915368209563547</v>
+        <v>0.00013915368209564504</v>
       </c>
       <c r="H19">
-        <v>0.00013130352291067067</v>
+        <v>0.0001313035229106804</v>
       </c>
       <c r="I19">
-        <v>9.1079901964059986e-05</v>
+        <v>9.1079901964069663e-05</v>
       </c>
       <c r="J19">
-        <v>6.999213058396495e-05</v>
+        <v>6.999213058397506e-05</v>
       </c>
       <c r="K19">
-        <v>0.00063230654186255972</v>
+        <v>0.00063230654186256547</v>
       </c>
       <c r="L19">
-        <v>0.00047289903568890847</v>
+        <v>0.00047289903568891465</v>
       </c>
       <c r="M19">
-        <v>-0.00021872529679949171</v>
+        <v>-0.00021872529679949068</v>
       </c>
       <c r="N19">
-        <v>-2.4394818592365961e-05</v>
+        <v>-2.4394818592364416e-05</v>
       </c>
       <c r="O19">
-        <v>2.4679496354268625e-05</v>
+        <v>2.4679496354270889e-05</v>
       </c>
       <c r="P19">
-        <v>-0.00011777917643881022</v>
+        <v>-0.00011777917643879086</v>
       </c>
       <c r="Q19">
-        <v>-0.00019017400239543304</v>
+        <v>-0.00019017400239541336</v>
       </c>
       <c r="R19">
-        <v>-0.00015611331133342095</v>
+        <v>-0.00015611331133340083</v>
       </c>
       <c r="S19">
-        <v>-0.00021038681129576778</v>
+        <v>-0.00021038681129574739</v>
       </c>
       <c r="T19">
-        <v>0.0010828886397138773</v>
+        <v>0.0010828886397138793</v>
       </c>
       <c r="U19">
-        <v>0.00095411326157021029</v>
+        <v>0.00095411326157021181</v>
       </c>
       <c r="V19">
-        <v>0.0009969685137757589</v>
+        <v>0.00099696851377575717</v>
       </c>
       <c r="W19">
-        <v>0.0010934520904993467</v>
+        <v>0.0010934520904993556</v>
       </c>
       <c r="X19">
-        <v>-9.7975365989235442e-05</v>
+        <v>-9.7975365989235293e-05</v>
       </c>
       <c r="Y19">
-        <v>6.9257082614885125e-06</v>
+        <v>6.9257082614884854e-06</v>
       </c>
       <c r="Z19">
-        <v>5.8451861510897723e-05</v>
+        <v>5.8451861510900867e-05</v>
       </c>
       <c r="AA19">
-        <v>5.2488330671794366e-05</v>
+        <v>5.2488330671796534e-05</v>
       </c>
       <c r="AB19">
-        <v>2.1032802931347859e-05</v>
+        <v>2.1032802931350678e-05</v>
       </c>
       <c r="AC19">
-        <v>3.3098360869946624e-05</v>
+        <v>3.3098360869949768e-05</v>
       </c>
       <c r="AD19">
-        <v>2.1061296049569659e-05</v>
+        <v>2.1061296049572695e-05</v>
       </c>
       <c r="AE19">
-        <v>0.00011004290423317754</v>
+        <v>0.0001100429042331806</v>
       </c>
       <c r="AF19">
-        <v>-3.1269371662587711e-06</v>
+        <v>-3.1269371662585882e-06</v>
       </c>
       <c r="AG19">
-        <v>-0.00013761921847101522</v>
+        <v>-0.00013761921847101533</v>
       </c>
       <c r="AH19">
-        <v>-5.2297174353573331e-05</v>
+        <v>-5.2297174353574253e-05</v>
       </c>
       <c r="AI19">
-        <v>-0.00073223072105569578</v>
+        <v>-0.00073223072105571747</v>
       </c>
     </row>
     <row r="20">
@@ -2431,103 +2431,103 @@
         <v>0.079518653485038435</v>
       </c>
       <c r="C20">
-        <v>3.897800193710734e-05</v>
+        <v>3.8978001937107882e-05</v>
       </c>
       <c r="D20">
-        <v>-3.2793598063826689e-05</v>
+        <v>-3.2793598063814329e-05</v>
       </c>
       <c r="E20">
-        <v>9.0123156531705896e-05</v>
+        <v>9.0123156531717605e-05</v>
       </c>
       <c r="F20">
-        <v>4.759201680919038e-05</v>
+        <v>4.7592016809201655e-05</v>
       </c>
       <c r="G20">
-        <v>0.00021119581025745267</v>
+        <v>0.00021119581025746525</v>
       </c>
       <c r="H20">
-        <v>0.00014664378215088975</v>
+        <v>0.00014664378215090254</v>
       </c>
       <c r="I20">
-        <v>0.00022175602752184205</v>
+        <v>0.00022175602752185462</v>
       </c>
       <c r="J20">
-        <v>7.925130788153387e-05</v>
+        <v>7.9251307881547098e-05</v>
       </c>
       <c r="K20">
-        <v>0.0032118980277105877</v>
+        <v>0.0032118980277105924</v>
       </c>
       <c r="L20">
-        <v>0.0026454966364136681</v>
+        <v>0.002645496636413675</v>
       </c>
       <c r="M20">
-        <v>-0.00055939481065233362</v>
+        <v>-0.00055939481065233254</v>
       </c>
       <c r="N20">
-        <v>0.00014571898141819267</v>
+        <v>0.00014571898141819425</v>
       </c>
       <c r="O20">
-        <v>0.00018782629432656083</v>
+        <v>0.00018782629432656311</v>
       </c>
       <c r="P20">
-        <v>0.00038688893363880315</v>
+        <v>0.00038688893363882744</v>
       </c>
       <c r="Q20">
-        <v>-2.4202738745484134e-07</v>
+        <v>-2.4202738742925417e-07</v>
       </c>
       <c r="R20">
-        <v>6.7493561899841393e-05</v>
+        <v>6.7493561899867414e-05</v>
       </c>
       <c r="S20">
-        <v>0.00017642226562673922</v>
+        <v>0.0001764222656267648</v>
       </c>
       <c r="T20">
-        <v>0.00095411326157021029</v>
+        <v>0.00095411326157021181</v>
       </c>
       <c r="U20">
-        <v>0.0035249377378211919</v>
+        <v>0.0035249377378211962</v>
       </c>
       <c r="V20">
-        <v>0.0033561089904270564</v>
+        <v>0.0033561089904270485</v>
       </c>
       <c r="W20">
-        <v>0.0036402634101280343</v>
+        <v>0.0036402634101280655</v>
       </c>
       <c r="X20">
-        <v>-0.0002085859767480611</v>
+        <v>-0.00020858597674806067</v>
       </c>
       <c r="Y20">
-        <v>2.5943844974372215e-05</v>
+        <v>2.5943844974371945e-05</v>
       </c>
       <c r="Z20">
-        <v>2.768071263798029e-05</v>
+        <v>2.7680712637990265e-05</v>
       </c>
       <c r="AA20">
-        <v>-2.6550282929700686e-05</v>
+        <v>-2.6550282929693313e-05</v>
       </c>
       <c r="AB20">
-        <v>-3.9589942205490092e-05</v>
+        <v>-3.9589942205481418e-05</v>
       </c>
       <c r="AC20">
-        <v>4.6144882518512828e-06</v>
+        <v>4.6144882518608238e-06</v>
       </c>
       <c r="AD20">
-        <v>0.0001070700554739681</v>
+        <v>0.00010707005547397802</v>
       </c>
       <c r="AE20">
-        <v>7.5686072508696781e-05</v>
+        <v>7.5686072508706647e-05</v>
       </c>
       <c r="AF20">
-        <v>4.5265732748416096e-06</v>
+        <v>4.5265732748422195e-06</v>
       </c>
       <c r="AG20">
-        <v>-2.3809894667179386e-05</v>
+        <v>-2.3809894667178953e-05</v>
       </c>
       <c r="AH20">
-        <v>-6.8373762652340847e-05</v>
+        <v>-6.83737626523441e-05</v>
       </c>
       <c r="AI20">
-        <v>-0.0036109294228694145</v>
+        <v>-0.0036109294228694813</v>
       </c>
     </row>
     <row r="21">
@@ -2538,103 +2538,103 @@
         <v>0.20038459830311944</v>
       </c>
       <c r="C21">
-        <v>-1.429762836629479e-06</v>
+        <v>-1.4297628366294248e-06</v>
       </c>
       <c r="D21">
-        <v>0.00034904637853419248</v>
+        <v>0.00034904637853420397</v>
       </c>
       <c r="E21">
-        <v>0.00023564401616686876</v>
+        <v>0.00023564401616688263</v>
       </c>
       <c r="F21">
-        <v>6.0529809378991268e-05</v>
+        <v>6.0529809379003194e-05</v>
       </c>
       <c r="G21">
-        <v>0.00054653907747107444</v>
+        <v>0.00054653907747108572</v>
       </c>
       <c r="H21">
-        <v>0.00051188472275484316</v>
+        <v>0.00051188472275485487</v>
       </c>
       <c r="I21">
-        <v>0.0003513849927976253</v>
+        <v>0.00035138499279763918</v>
       </c>
       <c r="J21">
-        <v>0.0004394237064820612</v>
+        <v>0.00043942370648207335</v>
       </c>
       <c r="K21">
-        <v>0.0036789130441664463</v>
+        <v>0.0036789130441664351</v>
       </c>
       <c r="L21">
-        <v>0.0030849932598246382</v>
+        <v>0.0030849932598246296</v>
       </c>
       <c r="M21">
-        <v>-0.00045654085313738161</v>
+        <v>-0.00045654085313738102</v>
       </c>
       <c r="N21">
-        <v>0.00024170927075665868</v>
+        <v>0.00024170927075665923</v>
       </c>
       <c r="O21">
-        <v>0.00029188576739535427</v>
+        <v>0.00029188576739535514</v>
       </c>
       <c r="P21">
-        <v>0.00055400873771308933</v>
+        <v>0.00055400873771309887</v>
       </c>
       <c r="Q21">
-        <v>-2.6207257167606968e-05</v>
+        <v>-2.6207257167597427e-05</v>
       </c>
       <c r="R21">
-        <v>-1.1335263924642028e-05</v>
+        <v>-1.1335263924633354e-05</v>
       </c>
       <c r="S21">
-        <v>0.00013642230501540332</v>
+        <v>0.00013642230501541286</v>
       </c>
       <c r="T21">
-        <v>0.0009969685137757589</v>
+        <v>0.00099696851377575717</v>
       </c>
       <c r="U21">
-        <v>0.0033561089904270564</v>
+        <v>0.0033561089904270485</v>
       </c>
       <c r="V21">
-        <v>0.0044746450417367783</v>
+        <v>0.0044746450417367679</v>
       </c>
       <c r="W21">
-        <v>0.0042381389294276536</v>
+        <v>0.0042381389294276935</v>
       </c>
       <c r="X21">
-        <v>-0.00021322219030547236</v>
+        <v>-0.00021322219030547171</v>
       </c>
       <c r="Y21">
-        <v>2.7666029659508765e-05</v>
+        <v>2.7666029659508548e-05</v>
       </c>
       <c r="Z21">
-        <v>8.6603241043895548e-05</v>
+        <v>8.6603241043908558e-05</v>
       </c>
       <c r="AA21">
-        <v>1.9365119552465504e-06</v>
+        <v>1.9365119552565251e-06</v>
       </c>
       <c r="AB21">
-        <v>3.0966175405273098e-05</v>
+        <v>3.0966175405284808e-05</v>
       </c>
       <c r="AC21">
-        <v>7.6567174047375945e-05</v>
+        <v>7.6567174047388088e-05</v>
       </c>
       <c r="AD21">
-        <v>0.00018787443626774088</v>
+        <v>0.00018787443626775379</v>
       </c>
       <c r="AE21">
-        <v>0.00020760721124195796</v>
+        <v>0.00020760721124197113</v>
       </c>
       <c r="AF21">
-        <v>9.0116810501175454e-06</v>
+        <v>9.0116810501183992e-06</v>
       </c>
       <c r="AG21">
         <v>9.8761563418469159e-05</v>
       </c>
       <c r="AH21">
-        <v>-0.00010339082551956988</v>
+        <v>-0.00010339082551957465</v>
       </c>
       <c r="AI21">
-        <v>-0.0044241714089441721</v>
+        <v>-0.0044241714089442597</v>
       </c>
     </row>
     <row r="22">
@@ -2645,103 +2645,103 @@
         <v>0.23388741978217065</v>
       </c>
       <c r="C22">
-        <v>-5.9422502834602001e-05</v>
+        <v>-5.9422502834600118e-05</v>
       </c>
       <c r="D22">
-        <v>0.00080519745304555952</v>
+        <v>0.000805197453045594</v>
       </c>
       <c r="E22">
-        <v>0.00072939579332476838</v>
+        <v>0.0007293957933247996</v>
       </c>
       <c r="F22">
-        <v>0.00035402050081689601</v>
+        <v>0.00035402050081692485</v>
       </c>
       <c r="G22">
-        <v>0.0012059413454082234</v>
+        <v>0.0012059413454082583</v>
       </c>
       <c r="H22">
-        <v>0.001063574258902799</v>
+        <v>0.0010635742589028341</v>
       </c>
       <c r="I22">
-        <v>0.000769543349896985</v>
+        <v>0.00076954334989701731</v>
       </c>
       <c r="J22">
-        <v>0.00077552129634346251</v>
+        <v>0.00077552129634349829</v>
       </c>
       <c r="K22">
-        <v>0.0039392190568509015</v>
+        <v>0.0039392190568509327</v>
       </c>
       <c r="L22">
-        <v>0.0033259568499667243</v>
+        <v>0.003325956849966759</v>
       </c>
       <c r="M22">
-        <v>-0.00033281241228975955</v>
+        <v>-0.00033281241228975544</v>
       </c>
       <c r="N22">
-        <v>0.00043867877034087726</v>
+        <v>0.00043867877034088393</v>
       </c>
       <c r="O22">
-        <v>0.00050573604431693045</v>
+        <v>0.00050573604431693945</v>
       </c>
       <c r="P22">
-        <v>0.00046371833807942004</v>
+        <v>0.00046371833807950721</v>
       </c>
       <c r="Q22">
-        <v>1.6812808064698651e-05</v>
+        <v>1.6812808064787556e-05</v>
       </c>
       <c r="R22">
-        <v>5.8702360032054837e-05</v>
+        <v>5.870236003214591e-05</v>
       </c>
       <c r="S22">
-        <v>0.00025997622043381517</v>
+        <v>0.00025997622043390668</v>
       </c>
       <c r="T22">
-        <v>0.0010934520904993467</v>
+        <v>0.0010934520904993556</v>
       </c>
       <c r="U22">
-        <v>0.0036402634101280343</v>
+        <v>0.0036402634101280655</v>
       </c>
       <c r="V22">
-        <v>0.0042381389294276536</v>
+        <v>0.0042381389294276935</v>
       </c>
       <c r="W22">
-        <v>0.0054224935541577687</v>
+        <v>0.005422493554157819</v>
       </c>
       <c r="X22">
-        <v>-0.00025246361274046842</v>
+        <v>-0.00025246361274046782</v>
       </c>
       <c r="Y22">
-        <v>2.9979686537174189e-05</v>
+        <v>2.9979686537174081e-05</v>
       </c>
       <c r="Z22">
-        <v>0.00016191570019673729</v>
+        <v>0.00016191570019675463</v>
       </c>
       <c r="AA22">
-        <v>2.6869125629069759e-05</v>
+        <v>2.6869125629082336e-05</v>
       </c>
       <c r="AB22">
-        <v>5.4205815082350884e-05</v>
+        <v>5.4205815082366497e-05</v>
       </c>
       <c r="AC22">
-        <v>0.00013184405026467035</v>
+        <v>0.0001318440502646864</v>
       </c>
       <c r="AD22">
-        <v>0.00019495295271682251</v>
+        <v>0.00019495295271683931</v>
       </c>
       <c r="AE22">
-        <v>0.00014314395619293653</v>
+        <v>0.00014314395619295401</v>
       </c>
       <c r="AF22">
-        <v>1.1770680230066018e-05</v>
+        <v>1.1770680230067129e-05</v>
       </c>
       <c r="AG22">
-        <v>-0.00017259147849396899</v>
+        <v>-0.00017259147849397072</v>
       </c>
       <c r="AH22">
-        <v>-0.00014225457160009481</v>
+        <v>-0.00014225457160010066</v>
       </c>
       <c r="AI22">
-        <v>-0.0053221193019862469</v>
+        <v>-0.0053221193019863666</v>
       </c>
     </row>
     <row r="23">
@@ -2752,103 +2752,103 @@
         <v>0.01736585391862102</v>
       </c>
       <c r="C23">
-        <v>-4.802813257907438e-07</v>
+        <v>-4.8028132579072198e-07</v>
       </c>
       <c r="D23">
-        <v>-7.8230614138234162e-06</v>
+        <v>-7.8230614138232163e-06</v>
       </c>
       <c r="E23">
-        <v>-3.1864712784610305e-05</v>
+        <v>-3.1864712784610176e-05</v>
       </c>
       <c r="F23">
-        <v>-1.1239453734116289e-05</v>
+        <v>-1.1239453734116243e-05</v>
       </c>
       <c r="G23">
-        <v>-4.7557013707125948e-05</v>
+        <v>-4.7557013707125826e-05</v>
       </c>
       <c r="H23">
-        <v>-2.6566527801927502e-05</v>
+        <v>-2.6566527801927329e-05</v>
       </c>
       <c r="I23">
-        <v>-3.6324449322708719e-05</v>
+        <v>-3.6324449322708611e-05</v>
       </c>
       <c r="J23">
-        <v>-3.8749522387691831e-05</v>
+        <v>-3.8749522387691655e-05</v>
       </c>
       <c r="K23">
-        <v>-0.00016679003225496483</v>
+        <v>-0.00016679003225496437</v>
       </c>
       <c r="L23">
-        <v>-0.0001492195673697877</v>
+        <v>-0.00014921956736978716</v>
       </c>
       <c r="M23">
-        <v>1.3508018690001934e-05</v>
+        <v>1.3508018690001983e-05</v>
       </c>
       <c r="N23">
-        <v>-8.9450452029444165e-06</v>
+        <v>-8.94504520294432e-06</v>
       </c>
       <c r="O23">
-        <v>-1.0285577321125531e-05</v>
+        <v>-1.0285577321125419e-05</v>
       </c>
       <c r="P23">
-        <v>-2.9039404761879379e-05</v>
+        <v>-2.9039404761877563e-05</v>
       </c>
       <c r="Q23">
-        <v>-1.5446679067544567e-05</v>
+        <v>-1.5446679067542744e-05</v>
       </c>
       <c r="R23">
-        <v>-1.4914311524460619e-05</v>
+        <v>-1.4914311524458736e-05</v>
       </c>
       <c r="S23">
-        <v>-1.2964826891340041e-05</v>
+        <v>-1.2964826891338069e-05</v>
       </c>
       <c r="T23">
-        <v>-9.7975365989235442e-05</v>
+        <v>-9.7975365989235293e-05</v>
       </c>
       <c r="U23">
-        <v>-0.0002085859767480611</v>
+        <v>-0.00020858597674806067</v>
       </c>
       <c r="V23">
-        <v>-0.00021322219030547236</v>
+        <v>-0.00021322219030547171</v>
       </c>
       <c r="W23">
-        <v>-0.00025246361274046842</v>
+        <v>-0.00025246361274046782</v>
       </c>
       <c r="X23">
-        <v>3.5907221896566375e-05</v>
+        <v>3.5907221896566362e-05</v>
       </c>
       <c r="Y23">
-        <v>-5.0879498333561162e-06</v>
+        <v>-5.0879498333560857e-06</v>
       </c>
       <c r="Z23">
-        <v>-1.4893099836860317e-05</v>
+        <v>-1.4893099836860914e-05</v>
       </c>
       <c r="AA23">
-        <v>-1.3096336156970693e-05</v>
+        <v>-1.3096336156971045e-05</v>
       </c>
       <c r="AB23">
-        <v>-7.4033122276246515e-06</v>
+        <v>-7.4033122276251123e-06</v>
       </c>
       <c r="AC23">
-        <v>-1.2136815108224061e-05</v>
+        <v>-1.2136815108224671e-05</v>
       </c>
       <c r="AD23">
-        <v>-8.7635720959443405e-06</v>
+        <v>-8.7635720959448961e-06</v>
       </c>
       <c r="AE23">
-        <v>-1.5430911525350005e-05</v>
+        <v>-1.5430911525350564e-05</v>
       </c>
       <c r="AF23">
-        <v>1.9760107536395215e-06</v>
+        <v>1.9760107536394927e-06</v>
       </c>
       <c r="AG23">
-        <v>3.0246414570963748e-05</v>
+        <v>3.0246414570963667e-05</v>
       </c>
       <c r="AH23">
-        <v>-4.9263320160389701e-06</v>
+        <v>-4.9263320160388346e-06</v>
       </c>
       <c r="AI23">
-        <v>0.00018792114322453663</v>
+        <v>0.0001879211432245401</v>
       </c>
     </row>
     <row r="24">
@@ -2859,103 +2859,103 @@
         <v>3.892237300748834</v>
       </c>
       <c r="C24">
-        <v>-3.1834493471115892e-05</v>
+        <v>-3.1834493471115865e-05</v>
       </c>
       <c r="D24">
-        <v>0.00033228372241895826</v>
+        <v>0.00033228372241895908</v>
       </c>
       <c r="E24">
-        <v>-6.7136134926304263e-05</v>
+        <v>-6.7136134926303558e-05</v>
       </c>
       <c r="F24">
-        <v>-4.883454486433441e-05</v>
+        <v>-4.883454486433376e-05</v>
       </c>
       <c r="G24">
-        <v>0.00012877618346038923</v>
+        <v>0.00012877618346038988</v>
       </c>
       <c r="H24">
-        <v>-1.8494888706545559e-05</v>
+        <v>-1.8494888706544908e-05</v>
       </c>
       <c r="I24">
-        <v>-8.8974886706919552e-05</v>
+        <v>-8.8974886706918684e-05</v>
       </c>
       <c r="J24">
-        <v>-2.3845104977733469e-05</v>
+        <v>-2.384510497773271e-05</v>
       </c>
       <c r="K24">
-        <v>3.7762544182087083e-05</v>
+        <v>3.7762544182086649e-05</v>
       </c>
       <c r="L24">
-        <v>4.2739638244125274e-05</v>
+        <v>4.2739638244124894e-05</v>
       </c>
       <c r="M24">
-        <v>3.3516023083526297e-06</v>
+        <v>3.3516023083527584e-06</v>
       </c>
       <c r="N24">
-        <v>2.5349901746122248e-06</v>
+        <v>2.5349901746123875e-06</v>
       </c>
       <c r="O24">
-        <v>1.0451598659236535e-05</v>
+        <v>1.0451598659236752e-05</v>
       </c>
       <c r="P24">
-        <v>-0.00011733515753141401</v>
+        <v>-0.00011733515753141271</v>
       </c>
       <c r="Q24">
-        <v>-2.0611295039211402e-05</v>
+        <v>-2.0611295039210317e-05</v>
       </c>
       <c r="R24">
-        <v>-2.791809035572186e-05</v>
+        <v>-2.7918090355720342e-05</v>
       </c>
       <c r="S24">
-        <v>1.2286128425974523e-06</v>
+        <v>1.2286128425987534e-06</v>
       </c>
       <c r="T24">
-        <v>6.9257082614885125e-06</v>
+        <v>6.9257082614884854e-06</v>
       </c>
       <c r="U24">
-        <v>2.5943844974372215e-05</v>
+        <v>2.5943844974371945e-05</v>
       </c>
       <c r="V24">
-        <v>2.7666029659508765e-05</v>
+        <v>2.7666029659508548e-05</v>
       </c>
       <c r="W24">
-        <v>2.9979686537174189e-05</v>
+        <v>2.9979686537174081e-05</v>
       </c>
       <c r="X24">
-        <v>-5.0879498333561162e-06</v>
+        <v>-5.0879498333560857e-06</v>
       </c>
       <c r="Y24">
         <v>0.00046673961194149469</v>
       </c>
       <c r="Z24">
-        <v>-1.3656190882247636e-05</v>
+        <v>-1.3656190882247501e-05</v>
       </c>
       <c r="AA24">
-        <v>2.3027779609006551e-05</v>
+        <v>2.3027779609006741e-05</v>
       </c>
       <c r="AB24">
-        <v>-1.2590197192875486e-05</v>
+        <v>-1.2590197192875337e-05</v>
       </c>
       <c r="AC24">
-        <v>-5.4273072590255015e-06</v>
+        <v>-5.4273072590252304e-06</v>
       </c>
       <c r="AD24">
-        <v>5.0475275273062659e-06</v>
+        <v>5.0475275273064929e-06</v>
       </c>
       <c r="AE24">
-        <v>-4.6852151554368798e-05</v>
+        <v>-4.6852151554368649e-05</v>
       </c>
       <c r="AF24">
-        <v>-1.5188203201894497e-07</v>
+        <v>-1.5188203201892972e-07</v>
       </c>
       <c r="AG24">
-        <v>-0.00010559568546626718</v>
+        <v>-0.00010559568546626726</v>
       </c>
       <c r="AH24">
-        <v>2.8898995698168813e-05</v>
+        <v>2.8898995698168637e-05</v>
       </c>
       <c r="AI24">
-        <v>-0.00018355116897700159</v>
+        <v>-0.00018355116897699833</v>
       </c>
     </row>
     <row r="25">
@@ -2966,103 +2966,103 @@
         <v>0.094379236628785945</v>
       </c>
       <c r="C25">
-        <v>-8.1085924364915341e-05</v>
+        <v>-8.1085924364914826e-05</v>
       </c>
       <c r="D25">
-        <v>0.00014280146279554637</v>
+        <v>0.00014280146279555895</v>
       </c>
       <c r="E25">
-        <v>0.00010394145986337652</v>
+        <v>0.00010394145986338931</v>
       </c>
       <c r="F25">
-        <v>0.00011191749201079561</v>
+        <v>0.00011191749201080623</v>
       </c>
       <c r="G25">
-        <v>0.00020423090026065174</v>
+        <v>0.00020423090026066562</v>
       </c>
       <c r="H25">
-        <v>0.00022190153581250639</v>
+        <v>0.00022190153581251983</v>
       </c>
       <c r="I25">
-        <v>5.285445932202786e-05</v>
+        <v>5.2854459322041088e-05</v>
       </c>
       <c r="J25">
-        <v>0.00014993704661024967</v>
+        <v>0.00014993704661026355</v>
       </c>
       <c r="K25">
-        <v>0.00018681899800963376</v>
+        <v>0.0001868189980096433</v>
       </c>
       <c r="L25">
-        <v>4.4432803402145657e-05</v>
+        <v>4.4432803402155632e-05</v>
       </c>
       <c r="M25">
-        <v>5.3753552470530829e-06</v>
+        <v>5.3753552470534624e-06</v>
       </c>
       <c r="N25">
-        <v>3.176840152891992e-05</v>
+        <v>3.176840152892095e-05</v>
       </c>
       <c r="O25">
-        <v>7.8399976348818355e-05</v>
+        <v>7.8399976348820632e-05</v>
       </c>
       <c r="P25">
-        <v>0.00011420262847560651</v>
+        <v>0.00011420262847562559</v>
       </c>
       <c r="Q25">
-        <v>0.00039977578339571874</v>
+        <v>0.00039977578339573782</v>
       </c>
       <c r="R25">
-        <v>0.00042834881384021077</v>
+        <v>0.00042834881384023072</v>
       </c>
       <c r="S25">
-        <v>0.00050815612522661473</v>
+        <v>0.00050815612522663554</v>
       </c>
       <c r="T25">
-        <v>5.8451861510897723e-05</v>
+        <v>5.8451861510900867e-05</v>
       </c>
       <c r="U25">
-        <v>2.768071263798029e-05</v>
+        <v>2.7680712637990265e-05</v>
       </c>
       <c r="V25">
-        <v>8.6603241043895548e-05</v>
+        <v>8.6603241043908558e-05</v>
       </c>
       <c r="W25">
-        <v>0.00016191570019673729</v>
+        <v>0.00016191570019675463</v>
       </c>
       <c r="X25">
-        <v>-1.4893099836860317e-05</v>
+        <v>-1.4893099836860914e-05</v>
       </c>
       <c r="Y25">
-        <v>-1.3656190882247636e-05</v>
+        <v>-1.3656190882247501e-05</v>
       </c>
       <c r="Z25">
-        <v>0.0030697965617201852</v>
+        <v>0.00306979656172019</v>
       </c>
       <c r="AA25">
-        <v>0.0024179089040784613</v>
+        <v>0.0024179089040784673</v>
       </c>
       <c r="AB25">
-        <v>0.002404550751804479</v>
+        <v>0.0024045507518044842</v>
       </c>
       <c r="AC25">
-        <v>0.0024220989664617064</v>
+        <v>0.002422098966461712</v>
       </c>
       <c r="AD25">
-        <v>0.0024195156018215242</v>
+        <v>0.0024195156018215289</v>
       </c>
       <c r="AE25">
-        <v>0.0024034528561093405</v>
+        <v>0.0024034528561093466</v>
       </c>
       <c r="AF25">
-        <v>4.3270358777724812e-06</v>
+        <v>4.3270358777728335e-06</v>
       </c>
       <c r="AG25">
-        <v>-8.9653440550173033e-05</v>
+        <v>-8.9653440550173901e-05</v>
       </c>
       <c r="AH25">
-        <v>-7.5214449039279706e-05</v>
+        <v>-7.5214449039282634e-05</v>
       </c>
       <c r="AI25">
-        <v>-0.0030368046871220981</v>
+        <v>-0.0030368046871221436</v>
       </c>
     </row>
     <row r="26">
@@ -3073,103 +3073,103 @@
         <v>0.12294840072921695</v>
       </c>
       <c r="C26">
-        <v>-8.7021960423897996e-05</v>
+        <v>-8.7021960423897508e-05</v>
       </c>
       <c r="D26">
-        <v>0.0010716454027064866</v>
+        <v>0.0010716454027064983</v>
       </c>
       <c r="E26">
-        <v>8.770373819365785e-05</v>
+        <v>8.7703738193669126e-05</v>
       </c>
       <c r="F26">
-        <v>7.3842847933200395e-06</v>
+        <v>7.3842847933297973e-06</v>
       </c>
       <c r="G26">
-        <v>6.1444208924456853e-05</v>
+        <v>6.1444208924468779e-05</v>
       </c>
       <c r="H26">
-        <v>0.00014698745143087479</v>
+        <v>0.00014698745143088671</v>
       </c>
       <c r="I26">
-        <v>3.2123447875525299e-05</v>
+        <v>3.2123447875537442e-05</v>
       </c>
       <c r="J26">
-        <v>0.00012300481935884349</v>
+        <v>0.00012300481935885563</v>
       </c>
       <c r="K26">
-        <v>0.00010292825587060895</v>
+        <v>0.00010292825587061589</v>
       </c>
       <c r="L26">
-        <v>-5.0739540888786183e-05</v>
+        <v>-5.0739540888778811e-05</v>
       </c>
       <c r="M26">
-        <v>-4.7040608925575636e-05</v>
+        <v>-4.7040608925574498e-05</v>
       </c>
       <c r="N26">
-        <v>1.4427976619051325e-05</v>
+        <v>1.4427976619053114e-05</v>
       </c>
       <c r="O26">
-        <v>8.0597869771119454e-05</v>
+        <v>8.0597869771121947e-05</v>
       </c>
       <c r="P26">
-        <v>0.00016597672273013959</v>
+        <v>0.00016597672273016388</v>
       </c>
       <c r="Q26">
-        <v>0.00039619269341183844</v>
+        <v>0.00039619269341186359</v>
       </c>
       <c r="R26">
-        <v>0.00038964786848787094</v>
+        <v>0.00038964786848789609</v>
       </c>
       <c r="S26">
-        <v>0.00043808842808900489</v>
+        <v>0.00043808842808903178</v>
       </c>
       <c r="T26">
-        <v>5.2488330671794366e-05</v>
+        <v>5.2488330671796534e-05</v>
       </c>
       <c r="U26">
-        <v>-2.6550282929700686e-05</v>
+        <v>-2.6550282929693313e-05</v>
       </c>
       <c r="V26">
-        <v>1.9365119552465504e-06</v>
+        <v>1.9365119552565251e-06</v>
       </c>
       <c r="W26">
-        <v>2.6869125629069759e-05</v>
+        <v>2.6869125629082336e-05</v>
       </c>
       <c r="X26">
-        <v>-1.3096336156970693e-05</v>
+        <v>-1.3096336156971045e-05</v>
       </c>
       <c r="Y26">
-        <v>2.3027779609006551e-05</v>
+        <v>2.3027779609006741e-05</v>
       </c>
       <c r="Z26">
-        <v>0.0024179089040784613</v>
+        <v>0.0024179089040784673</v>
       </c>
       <c r="AA26">
-        <v>0.0031027946331042924</v>
+        <v>0.0031027946331042976</v>
       </c>
       <c r="AB26">
-        <v>0.0023978483286616562</v>
+        <v>0.0023978483286616614</v>
       </c>
       <c r="AC26">
-        <v>0.002409357967163568</v>
+        <v>0.0024093579671635732</v>
       </c>
       <c r="AD26">
-        <v>0.0024111185307734502</v>
+        <v>0.002411118530773455</v>
       </c>
       <c r="AE26">
-        <v>0.0024006466571823933</v>
+        <v>0.0024006466571823981</v>
       </c>
       <c r="AF26">
-        <v>5.2611654468122114e-06</v>
+        <v>5.2611654468125231e-06</v>
       </c>
       <c r="AG26">
-        <v>-8.5541095288291539e-05</v>
+        <v>-8.554109528829219e-05</v>
       </c>
       <c r="AH26">
-        <v>-1.6356704670957467e-05</v>
+        <v>-1.6356704670960178e-05</v>
       </c>
       <c r="AI26">
-        <v>-0.0029087018043451578</v>
+        <v>-0.0029087018043451977</v>
       </c>
     </row>
     <row r="27">
@@ -3180,103 +3180,103 @@
         <v>-0.042363738032216963</v>
       </c>
       <c r="C27">
-        <v>-9.2596972208624484e-05</v>
+        <v>-9.2596972208624809e-05</v>
       </c>
       <c r="D27">
-        <v>0.0007563371623317567</v>
+        <v>0.0007563371623317696</v>
       </c>
       <c r="E27">
-        <v>0.00010743254938749445</v>
+        <v>0.00010743254938750703</v>
       </c>
       <c r="F27">
-        <v>5.2590944147562577e-05</v>
+        <v>5.2590944147573203e-05</v>
       </c>
       <c r="G27">
-        <v>0.0001231085885548299</v>
+        <v>0.00012310858855484356</v>
       </c>
       <c r="H27">
-        <v>0.00017526084095628117</v>
+        <v>0.00017526084095629484</v>
       </c>
       <c r="I27">
-        <v>5.362024703079349e-05</v>
+        <v>5.3620247030806501e-05</v>
       </c>
       <c r="J27">
-        <v>7.6264365752959753e-05</v>
+        <v>7.6264365752973414e-05</v>
       </c>
       <c r="K27">
-        <v>7.9016028483066278e-05</v>
+        <v>7.9016028483075602e-05</v>
       </c>
       <c r="L27">
-        <v>-2.6403228015850705e-05</v>
+        <v>-2.6403228015840947e-05</v>
       </c>
       <c r="M27">
-        <v>2.4527032191439961e-05</v>
+        <v>2.4527032191441208e-05</v>
       </c>
       <c r="N27">
-        <v>4.8685890455250794e-06</v>
+        <v>4.8685890455269767e-06</v>
       </c>
       <c r="O27">
-        <v>0.00010319506017073969</v>
+        <v>0.0001031950601707424</v>
       </c>
       <c r="P27">
-        <v>0.00016024217855355183</v>
+        <v>0.00016024217855357525</v>
       </c>
       <c r="Q27">
-        <v>0.00039999263156205271</v>
+        <v>0.00039999263156207613</v>
       </c>
       <c r="R27">
-        <v>0.00039390262233660652</v>
+        <v>0.00039390262233663341</v>
       </c>
       <c r="S27">
-        <v>0.00045272675287770861</v>
+        <v>0.00045272675287773376</v>
       </c>
       <c r="T27">
-        <v>2.1032802931347859e-05</v>
+        <v>2.1032802931350678e-05</v>
       </c>
       <c r="U27">
-        <v>-3.9589942205490092e-05</v>
+        <v>-3.9589942205481418e-05</v>
       </c>
       <c r="V27">
-        <v>3.0966175405273098e-05</v>
+        <v>3.0966175405284808e-05</v>
       </c>
       <c r="W27">
-        <v>5.4205815082350884e-05</v>
+        <v>5.4205815082366497e-05</v>
       </c>
       <c r="X27">
-        <v>-7.4033122276246515e-06</v>
+        <v>-7.4033122276251123e-06</v>
       </c>
       <c r="Y27">
-        <v>-1.2590197192875486e-05</v>
+        <v>-1.2590197192875337e-05</v>
       </c>
       <c r="Z27">
-        <v>0.002404550751804479</v>
+        <v>0.0024045507518044842</v>
       </c>
       <c r="AA27">
-        <v>0.0023978483286616562</v>
+        <v>0.0023978483286616614</v>
       </c>
       <c r="AB27">
-        <v>0.0029016948845160947</v>
+        <v>0.0029016948845160995</v>
       </c>
       <c r="AC27">
-        <v>0.0023941358533534473</v>
+        <v>0.0023941358533534521</v>
       </c>
       <c r="AD27">
-        <v>0.002393188555904899</v>
+        <v>0.0023931885559049038</v>
       </c>
       <c r="AE27">
-        <v>0.0023926236367021038</v>
+        <v>0.002392623636702109</v>
       </c>
       <c r="AF27">
-        <v>2.0155216062572577e-06</v>
+        <v>2.0155216062575626e-06</v>
       </c>
       <c r="AG27">
-        <v>-6.419983764488252e-05</v>
+        <v>-6.419983764488317e-05</v>
       </c>
       <c r="AH27">
-        <v>-9.5198216619427263e-05</v>
+        <v>-9.5198216619429973e-05</v>
       </c>
       <c r="AI27">
-        <v>-0.0028667674330144039</v>
+        <v>-0.0028667674330144456</v>
       </c>
     </row>
     <row r="28">
@@ -3287,103 +3287,103 @@
         <v>0.05751555787790158</v>
       </c>
       <c r="C28">
-        <v>-0.00010856841590938738</v>
+        <v>-0.00010856841590938695</v>
       </c>
       <c r="D28">
-        <v>0.00013931877986970488</v>
+        <v>0.00013931877986971463</v>
       </c>
       <c r="E28">
-        <v>4.3360577271745913e-05</v>
+        <v>4.3360577271755454e-05</v>
       </c>
       <c r="F28">
-        <v>-2.1056099340477884e-05</v>
+        <v>-2.1056099340469427e-05</v>
       </c>
       <c r="G28">
-        <v>6.6073099431141315e-05</v>
+        <v>6.6073099431151507e-05</v>
       </c>
       <c r="H28">
-        <v>9.9242546054492892e-05</v>
+        <v>9.9242546054503084e-05</v>
       </c>
       <c r="I28">
-        <v>-1.5459636173135441e-05</v>
+        <v>-1.54596361731259e-05</v>
       </c>
       <c r="J28">
-        <v>7.7531048207134723e-05</v>
+        <v>7.7531048207145131e-05</v>
       </c>
       <c r="K28">
-        <v>0.0001535077105833311</v>
+        <v>0.00015350771058333999</v>
       </c>
       <c r="L28">
-        <v>2.9783468960469656e-05</v>
+        <v>2.9783468960480498e-05</v>
       </c>
       <c r="M28">
-        <v>-2.7358458102672961e-05</v>
+        <v>-2.7358458102671876e-05</v>
       </c>
       <c r="N28">
-        <v>1.6549667470975769e-05</v>
+        <v>1.6549667470977449e-05</v>
       </c>
       <c r="O28">
-        <v>1.7201678399737103e-05</v>
+        <v>1.7201678399739488e-05</v>
       </c>
       <c r="P28">
-        <v>0.00011097867444821892</v>
+        <v>0.00011097867444824234</v>
       </c>
       <c r="Q28">
-        <v>0.00032778991844844511</v>
+        <v>0.00032778991844847026</v>
       </c>
       <c r="R28">
-        <v>0.00031836766960773727</v>
+        <v>0.00031836766960776329</v>
       </c>
       <c r="S28">
-        <v>0.00038264462745451165</v>
+        <v>0.00038264462745453767</v>
       </c>
       <c r="T28">
-        <v>3.3098360869946624e-05</v>
+        <v>3.3098360869949768e-05</v>
       </c>
       <c r="U28">
-        <v>4.6144882518512828e-06</v>
+        <v>4.6144882518608238e-06</v>
       </c>
       <c r="V28">
-        <v>7.6567174047375945e-05</v>
+        <v>7.6567174047388088e-05</v>
       </c>
       <c r="W28">
-        <v>0.00013184405026467035</v>
+        <v>0.0001318440502646864</v>
       </c>
       <c r="X28">
-        <v>-1.2136815108224061e-05</v>
+        <v>-1.2136815108224671e-05</v>
       </c>
       <c r="Y28">
-        <v>-5.4273072590255015e-06</v>
+        <v>-5.4273072590252304e-06</v>
       </c>
       <c r="Z28">
-        <v>0.0024220989664617064</v>
+        <v>0.002422098966461712</v>
       </c>
       <c r="AA28">
-        <v>0.002409357967163568</v>
+        <v>0.0024093579671635732</v>
       </c>
       <c r="AB28">
-        <v>0.0023941358533534473</v>
+        <v>0.0023941358533534521</v>
       </c>
       <c r="AC28">
-        <v>0.0029680040026244256</v>
+        <v>0.0029680040026244308</v>
       </c>
       <c r="AD28">
-        <v>0.0024122865124234327</v>
+        <v>0.0024122865124234379</v>
       </c>
       <c r="AE28">
-        <v>0.0024099257746925127</v>
+        <v>0.0024099257746925183</v>
       </c>
       <c r="AF28">
-        <v>5.4268485730809757e-06</v>
+        <v>5.4268485730813349e-06</v>
       </c>
       <c r="AG28">
-        <v>-7.3490856489324399e-05</v>
+        <v>-7.3490856489324833e-05</v>
       </c>
       <c r="AH28">
-        <v>-6.1148263188881189e-05</v>
+        <v>-6.1148263188884225e-05</v>
       </c>
       <c r="AI28">
-        <v>-0.0028181773427799263</v>
+        <v>-0.0028181773427799692</v>
       </c>
     </row>
     <row r="29">
@@ -3394,103 +3394,103 @@
         <v>-0.072941401664601224</v>
       </c>
       <c r="C29">
-        <v>-6.3819334106375331e-05</v>
+        <v>-6.3819334106375602e-05</v>
       </c>
       <c r="D29">
-        <v>0.00013819997115470237</v>
+        <v>0.0001381999711547124</v>
       </c>
       <c r="E29">
-        <v>6.5902518832273212e-05</v>
+        <v>6.5902518832282645e-05</v>
       </c>
       <c r="F29">
-        <v>-5.3059972264982548e-06</v>
+        <v>-5.3059972264900691e-06</v>
       </c>
       <c r="G29">
-        <v>2.2334027506154791e-05</v>
+        <v>2.233402750616547e-05</v>
       </c>
       <c r="H29">
-        <v>0.00011251699848729887</v>
+        <v>0.00011251699848730922</v>
       </c>
       <c r="I29">
-        <v>3.2777159819301132e-05</v>
+        <v>3.2777159819310836e-05</v>
       </c>
       <c r="J29">
-        <v>0.00016385404757253771</v>
+        <v>0.00016385404757254807</v>
       </c>
       <c r="K29">
-        <v>0.00035701943319050699</v>
+        <v>0.00035701943319051686</v>
       </c>
       <c r="L29">
-        <v>0.00011865440852693141</v>
+        <v>0.00011865440852694214</v>
       </c>
       <c r="M29">
-        <v>-7.4634030212139476e-05</v>
+        <v>-7.4634030212138337e-05</v>
       </c>
       <c r="N29">
-        <v>1.0462524298719981e-05</v>
+        <v>1.0462524298721825e-05</v>
       </c>
       <c r="O29">
-        <v>6.7471731706362253e-05</v>
+        <v>6.7471731706364855e-05</v>
       </c>
       <c r="P29">
-        <v>0.00021100525375209183</v>
+        <v>0.00021100525375211568</v>
       </c>
       <c r="Q29">
-        <v>0.00040526383753041113</v>
+        <v>0.00040526383753043585</v>
       </c>
       <c r="R29">
-        <v>0.00039693324408751564</v>
+        <v>0.00039693324408754101</v>
       </c>
       <c r="S29">
-        <v>0.00049446962267037727</v>
+        <v>0.00049446962267040286</v>
       </c>
       <c r="T29">
-        <v>2.1061296049569659e-05</v>
+        <v>2.1061296049572695e-05</v>
       </c>
       <c r="U29">
-        <v>0.0001070700554739681</v>
+        <v>0.00010707005547397802</v>
       </c>
       <c r="V29">
-        <v>0.00018787443626774088</v>
+        <v>0.00018787443626775379</v>
       </c>
       <c r="W29">
-        <v>0.00019495295271682251</v>
+        <v>0.00019495295271683931</v>
       </c>
       <c r="X29">
-        <v>-8.7635720959443405e-06</v>
+        <v>-8.7635720959448961e-06</v>
       </c>
       <c r="Y29">
-        <v>5.0475275273062659e-06</v>
+        <v>5.0475275273064929e-06</v>
       </c>
       <c r="Z29">
-        <v>0.0024195156018215242</v>
+        <v>0.0024195156018215289</v>
       </c>
       <c r="AA29">
-        <v>0.0024111185307734502</v>
+        <v>0.002411118530773455</v>
       </c>
       <c r="AB29">
-        <v>0.002393188555904899</v>
+        <v>0.0023931885559049038</v>
       </c>
       <c r="AC29">
-        <v>0.0024122865124234327</v>
+        <v>0.0024122865124234379</v>
       </c>
       <c r="AD29">
-        <v>0.0027931079009252111</v>
+        <v>0.0027931079009252159</v>
       </c>
       <c r="AE29">
-        <v>0.0024091875765934519</v>
+        <v>0.0024091875765934576</v>
       </c>
       <c r="AF29">
-        <v>8.473941459985273e-07</v>
+        <v>8.4739414599884578e-07</v>
       </c>
       <c r="AG29">
-        <v>5.9676148105947688e-05</v>
+        <v>5.9676148105947038e-05</v>
       </c>
       <c r="AH29">
-        <v>-3.4783355698563088e-05</v>
+        <v>-3.4783355698565798e-05</v>
       </c>
       <c r="AI29">
-        <v>-0.0030305872269813412</v>
+        <v>-0.003030587226981382</v>
       </c>
     </row>
     <row r="30">
@@ -3501,103 +3501,103 @@
         <v>0.065751712427960879</v>
       </c>
       <c r="C30">
-        <v>-4.7641209485684455e-06</v>
+        <v>-4.7641209485679661e-06</v>
       </c>
       <c r="D30">
-        <v>2.6842920995643992e-05</v>
+        <v>2.6842920995656433e-05</v>
       </c>
       <c r="E30">
-        <v>-1.1316323787113696e-05</v>
+        <v>-1.1316323787101472e-05</v>
       </c>
       <c r="F30">
-        <v>-7.2812817573096904e-05</v>
+        <v>-7.2812817573086278e-05</v>
       </c>
       <c r="G30">
-        <v>-3.5116145501650625e-05</v>
+        <v>-3.5116145501637398e-05</v>
       </c>
       <c r="H30">
-        <v>-6.6641415073845887e-06</v>
+        <v>-6.664141507371497e-06</v>
       </c>
       <c r="I30">
-        <v>2.4805335383795338e-05</v>
+        <v>2.4805335383808186e-05</v>
       </c>
       <c r="J30">
-        <v>1.1865457425506851e-05</v>
+        <v>1.1865457425520377e-05</v>
       </c>
       <c r="K30">
-        <v>0.0002187728275894843</v>
+        <v>0.00021877282758949387</v>
       </c>
       <c r="L30">
-        <v>-5.003866963365614e-05</v>
+        <v>-5.0038669633645488e-05</v>
       </c>
       <c r="M30">
-        <v>-0.00015014202061696563</v>
+        <v>-0.00015014202061696452</v>
       </c>
       <c r="N30">
-        <v>-2.3821879086441338e-05</v>
+        <v>-2.3821879086439562e-05</v>
       </c>
       <c r="O30">
-        <v>1.4188838300472849e-05</v>
+        <v>1.4188838300475437e-05</v>
       </c>
       <c r="P30">
-        <v>0.00039010103324478698</v>
+        <v>0.0003901010332448111</v>
       </c>
       <c r="Q30">
-        <v>0.00037619705005900988</v>
+        <v>0.00037619705005903449</v>
       </c>
       <c r="R30">
-        <v>0.00041366543595435884</v>
+        <v>0.0004136654359543841</v>
       </c>
       <c r="S30">
-        <v>0.00032125317013082764</v>
+        <v>0.0003212531701308536</v>
       </c>
       <c r="T30">
-        <v>0.00011004290423317754</v>
+        <v>0.0001100429042331806</v>
       </c>
       <c r="U30">
-        <v>7.5686072508696781e-05</v>
+        <v>7.5686072508706647e-05</v>
       </c>
       <c r="V30">
-        <v>0.00020760721124195796</v>
+        <v>0.00020760721124197113</v>
       </c>
       <c r="W30">
-        <v>0.00014314395619293653</v>
+        <v>0.00014314395619295401</v>
       </c>
       <c r="X30">
-        <v>-1.5430911525350005e-05</v>
+        <v>-1.5430911525350564e-05</v>
       </c>
       <c r="Y30">
-        <v>-4.6852151554368798e-05</v>
+        <v>-4.6852151554368649e-05</v>
       </c>
       <c r="Z30">
-        <v>0.0024034528561093405</v>
+        <v>0.0024034528561093466</v>
       </c>
       <c r="AA30">
-        <v>0.0024006466571823933</v>
+        <v>0.0024006466571823981</v>
       </c>
       <c r="AB30">
-        <v>0.0023926236367021038</v>
+        <v>0.002392623636702109</v>
       </c>
       <c r="AC30">
-        <v>0.0024099257746925127</v>
+        <v>0.0024099257746925183</v>
       </c>
       <c r="AD30">
-        <v>0.0024091875765934519</v>
+        <v>0.0024091875765934576</v>
       </c>
       <c r="AE30">
-        <v>0.0030251089773792807</v>
+        <v>0.0030251089773792855</v>
       </c>
       <c r="AF30">
-        <v>2.9194340006780237e-06</v>
+        <v>2.9194340006783489e-06</v>
       </c>
       <c r="AG30">
-        <v>-4.3658362118767502e-06</v>
+        <v>-4.3658362118780512e-06</v>
       </c>
       <c r="AH30">
-        <v>-9.5541077437662171e-05</v>
+        <v>-9.5541077437664881e-05</v>
       </c>
       <c r="AI30">
-        <v>-0.0028833015366855784</v>
+        <v>-0.00288330153668562</v>
       </c>
     </row>
     <row r="31">
@@ -3608,103 +3608,103 @@
         <v>0.001711011159776669</v>
       </c>
       <c r="C31">
-        <v>-1.9497710287320405e-06</v>
+        <v>-1.9497710287320125e-06</v>
       </c>
       <c r="D31">
-        <v>-8.510155342639439e-06</v>
+        <v>-8.510155342638653e-06</v>
       </c>
       <c r="E31">
-        <v>5.5397297790903439e-06</v>
+        <v>5.5397297790910622e-06</v>
       </c>
       <c r="F31">
-        <v>2.3800320149084932e-06</v>
+        <v>2.3800320149091234e-06</v>
       </c>
       <c r="G31">
-        <v>1.0130120580751479e-05</v>
+        <v>1.0130120580752258e-05</v>
       </c>
       <c r="H31">
-        <v>1.4003597577924943e-05</v>
+        <v>1.4003597577925736e-05</v>
       </c>
       <c r="I31">
-        <v>2.8167527087327672e-06</v>
+        <v>2.8167527087335329e-06</v>
       </c>
       <c r="J31">
-        <v>2.2537754202507757e-06</v>
+        <v>2.2537754202515888e-06</v>
       </c>
       <c r="K31">
-        <v>-3.2565980408890923e-07</v>
+        <v>-3.2565980408828582e-07</v>
       </c>
       <c r="L31">
-        <v>1.0516857342269178e-05</v>
+        <v>1.0516857342269856e-05</v>
       </c>
       <c r="M31">
-        <v>1.4859872921433072e-05</v>
+        <v>1.4859872921433194e-05</v>
       </c>
       <c r="N31">
-        <v>5.616813985184142e-06</v>
+        <v>5.6168139851843385e-06</v>
       </c>
       <c r="O31">
-        <v>9.5812939870465262e-06</v>
+        <v>9.5812939870467515e-06</v>
       </c>
       <c r="P31">
-        <v>5.7254640730687004e-06</v>
+        <v>5.7254640730701912e-06</v>
       </c>
       <c r="Q31">
-        <v>-2.857098044788532e-07</v>
+        <v>-2.8570980447728111e-07</v>
       </c>
       <c r="R31">
-        <v>3.6208117601797146e-06</v>
+        <v>3.6208117601813138e-06</v>
       </c>
       <c r="S31">
-        <v>6.4351374456237591e-06</v>
+        <v>6.4351374456253854e-06</v>
       </c>
       <c r="T31">
-        <v>-3.1269371662587711e-06</v>
+        <v>-3.1269371662585882e-06</v>
       </c>
       <c r="U31">
-        <v>4.5265732748416096e-06</v>
+        <v>4.5265732748422195e-06</v>
       </c>
       <c r="V31">
-        <v>9.0116810501175454e-06</v>
+        <v>9.0116810501183992e-06</v>
       </c>
       <c r="W31">
-        <v>1.1770680230066018e-05</v>
+        <v>1.1770680230067129e-05</v>
       </c>
       <c r="X31">
-        <v>1.9760107536395215e-06</v>
+        <v>1.9760107536394927e-06</v>
       </c>
       <c r="Y31">
-        <v>-1.5188203201894497e-07</v>
+        <v>-1.5188203201892972e-07</v>
       </c>
       <c r="Z31">
-        <v>4.3270358777724812e-06</v>
+        <v>4.3270358777728335e-06</v>
       </c>
       <c r="AA31">
-        <v>5.2611654468122114e-06</v>
+        <v>5.2611654468125231e-06</v>
       </c>
       <c r="AB31">
-        <v>2.0155216062572577e-06</v>
+        <v>2.0155216062575626e-06</v>
       </c>
       <c r="AC31">
-        <v>5.4268485730809757e-06</v>
+        <v>5.4268485730813349e-06</v>
       </c>
       <c r="AD31">
-        <v>8.473941459985273e-07</v>
+        <v>8.4739414599884578e-07</v>
       </c>
       <c r="AE31">
-        <v>2.9194340006780237e-06</v>
+        <v>2.9194340006783489e-06</v>
       </c>
       <c r="AF31">
-        <v>4.7593550376573534e-06</v>
+        <v>4.7593550376573975e-06</v>
       </c>
       <c r="AG31">
-        <v>-7.1751980030202551e-06</v>
+        <v>-7.1751980030204448e-06</v>
       </c>
       <c r="AH31">
-        <v>-1.3480168463238869e-05</v>
+        <v>-1.3480168463239126e-05</v>
       </c>
       <c r="AI31">
-        <v>-0.00011321363707010669</v>
+        <v>-0.00011321363707010979</v>
       </c>
     </row>
     <row r="32">
@@ -3715,103 +3715,103 @@
         <v>-0.15251988705998118</v>
       </c>
       <c r="C32">
-        <v>8.2682461790918376e-05</v>
+        <v>8.2682461790918268e-05</v>
       </c>
       <c r="D32">
-        <v>5.4247913094004809e-05</v>
+        <v>5.4247913094002641e-05</v>
       </c>
       <c r="E32">
-        <v>-3.4781742681625188e-05</v>
+        <v>-3.478174268162779e-05</v>
       </c>
       <c r="F32">
-        <v>0.00011273175229523135</v>
+        <v>0.00011273175229523005</v>
       </c>
       <c r="G32">
-        <v>-0.00013755789499182453</v>
+        <v>-0.00013755789499182583</v>
       </c>
       <c r="H32">
-        <v>-8.6778641401065969e-05</v>
+        <v>-8.677864140106727e-05</v>
       </c>
       <c r="I32">
-        <v>4.6806591355737746e-06</v>
+        <v>4.6806591355711726e-06</v>
       </c>
       <c r="J32">
-        <v>0.00015386211925594567</v>
+        <v>0.00015386211925594393</v>
       </c>
       <c r="K32">
-        <v>0.00037063543131517608</v>
+        <v>0.00037063543131517695</v>
       </c>
       <c r="L32">
         <v>5.5955232594965317e-05</v>
       </c>
       <c r="M32">
-        <v>-0.00030833222323535297</v>
+        <v>-0.0003083322232353533</v>
       </c>
       <c r="N32">
-        <v>-9.8069252881486258e-05</v>
+        <v>-9.8069252881486746e-05</v>
       </c>
       <c r="O32">
-        <v>-8.9809283282528017e-05</v>
+        <v>-8.9809283282528667e-05</v>
       </c>
       <c r="P32">
-        <v>1.2088203191898579e-05</v>
+        <v>1.2088203191894242e-05</v>
       </c>
       <c r="Q32">
-        <v>4.3779515320177889e-05</v>
+        <v>4.3779515320172685e-05</v>
       </c>
       <c r="R32">
-        <v>4.5946337358625244e-05</v>
+        <v>4.594633735862351e-05</v>
       </c>
       <c r="S32">
-        <v>4.3708144531398943e-05</v>
+        <v>4.3708144531393739e-05</v>
       </c>
       <c r="T32">
-        <v>-0.00013761921847101522</v>
+        <v>-0.00013761921847101533</v>
       </c>
       <c r="U32">
-        <v>-2.3809894667179386e-05</v>
+        <v>-2.3809894667178953e-05</v>
       </c>
       <c r="V32">
         <v>9.8761563418469159e-05</v>
       </c>
       <c r="W32">
-        <v>-0.00017259147849396899</v>
+        <v>-0.00017259147849397072</v>
       </c>
       <c r="X32">
-        <v>3.0246414570963748e-05</v>
+        <v>3.0246414570963667e-05</v>
       </c>
       <c r="Y32">
-        <v>-0.00010559568546626718</v>
+        <v>-0.00010559568546626726</v>
       </c>
       <c r="Z32">
-        <v>-8.9653440550173033e-05</v>
+        <v>-8.9653440550173901e-05</v>
       </c>
       <c r="AA32">
-        <v>-8.5541095288291539e-05</v>
+        <v>-8.554109528829219e-05</v>
       </c>
       <c r="AB32">
-        <v>-6.419983764488252e-05</v>
+        <v>-6.419983764488317e-05</v>
       </c>
       <c r="AC32">
-        <v>-7.3490856489324399e-05</v>
+        <v>-7.3490856489324833e-05</v>
       </c>
       <c r="AD32">
-        <v>5.9676148105947688e-05</v>
+        <v>5.9676148105947038e-05</v>
       </c>
       <c r="AE32">
-        <v>-4.3658362118767502e-06</v>
+        <v>-4.3658362118780512e-06</v>
       </c>
       <c r="AF32">
-        <v>-7.1751980030202551e-06</v>
+        <v>-7.1751980030204448e-06</v>
       </c>
       <c r="AG32">
-        <v>0.0021902531402251324</v>
+        <v>0.0021902531402251328</v>
       </c>
       <c r="AH32">
-        <v>0.00014619121712923053</v>
+        <v>0.00014619121712923123</v>
       </c>
       <c r="AI32">
-        <v>7.4687898885440079e-06</v>
+        <v>7.4687898885519226e-06</v>
       </c>
     </row>
     <row r="33">
@@ -3822,103 +3822,103 @@
         <v>-0.045878343329260198</v>
       </c>
       <c r="C33">
-        <v>1.3097791130418853e-05</v>
+        <v>1.3097791130418568e-05</v>
       </c>
       <c r="D33">
-        <v>0.0013306349657106415</v>
+        <v>0.0013306349657106369</v>
       </c>
       <c r="E33">
-        <v>2.948272168971347e-05</v>
+        <v>2.9482721689708916e-05</v>
       </c>
       <c r="F33">
-        <v>7.0103091909831813e-05</v>
+        <v>7.0103091909827909e-05</v>
       </c>
       <c r="G33">
-        <v>7.9445070357428687e-05</v>
+        <v>7.94450703574237e-05</v>
       </c>
       <c r="H33">
-        <v>6.0970632979302688e-05</v>
+        <v>6.0970632979297701e-05</v>
       </c>
       <c r="I33">
-        <v>3.7243755954839588e-05</v>
+        <v>3.7243755954834818e-05</v>
       </c>
       <c r="J33">
-        <v>-2.3520691061540422e-05</v>
+        <v>-2.3520691061545192e-05</v>
       </c>
       <c r="K33">
-        <v>-9.4744370399680016e-05</v>
+        <v>-9.4744370399683486e-05</v>
       </c>
       <c r="L33">
-        <v>-2.7635679663996337e-05</v>
+        <v>-2.7635679664000023e-05</v>
       </c>
       <c r="M33">
-        <v>-4.2100416755658121e-05</v>
+        <v>-4.2100416755658744e-05</v>
       </c>
       <c r="N33">
-        <v>-3.6525377833204319e-05</v>
+        <v>-3.6525377833205295e-05</v>
       </c>
       <c r="O33">
-        <v>-7.0967816654567714e-05</v>
+        <v>-7.0967816654568961e-05</v>
       </c>
       <c r="P33">
-        <v>-4.9005125978268584e-05</v>
+        <v>-4.9005125978278993e-05</v>
       </c>
       <c r="Q33">
-        <v>2.3744716712641081e-05</v>
+        <v>2.3744716712629371e-05</v>
       </c>
       <c r="R33">
-        <v>2.3263439245871376e-05</v>
+        <v>2.3263439245859233e-05</v>
       </c>
       <c r="S33">
-        <v>7.8244783439976838e-05</v>
+        <v>7.8244783439965129e-05</v>
       </c>
       <c r="T33">
-        <v>-5.2297174353573331e-05</v>
+        <v>-5.2297174353574253e-05</v>
       </c>
       <c r="U33">
-        <v>-6.8373762652340847e-05</v>
+        <v>-6.83737626523441e-05</v>
       </c>
       <c r="V33">
-        <v>-0.00010339082551956988</v>
+        <v>-0.00010339082551957465</v>
       </c>
       <c r="W33">
-        <v>-0.00014225457160009481</v>
+        <v>-0.00014225457160010066</v>
       </c>
       <c r="X33">
-        <v>-4.9263320160389701e-06</v>
+        <v>-4.9263320160388346e-06</v>
       </c>
       <c r="Y33">
-        <v>2.8898995698168813e-05</v>
+        <v>2.8898995698168637e-05</v>
       </c>
       <c r="Z33">
-        <v>-7.5214449039279706e-05</v>
+        <v>-7.5214449039282634e-05</v>
       </c>
       <c r="AA33">
-        <v>-1.6356704670957467e-05</v>
+        <v>-1.6356704670960178e-05</v>
       </c>
       <c r="AB33">
-        <v>-9.5198216619427263e-05</v>
+        <v>-9.5198216619429973e-05</v>
       </c>
       <c r="AC33">
-        <v>-6.1148263188881189e-05</v>
+        <v>-6.1148263188884225e-05</v>
       </c>
       <c r="AD33">
-        <v>-3.4783355698563088e-05</v>
+        <v>-3.4783355698565798e-05</v>
       </c>
       <c r="AE33">
-        <v>-9.5541077437662171e-05</v>
+        <v>-9.5541077437664881e-05</v>
       </c>
       <c r="AF33">
-        <v>-1.3480168463238869e-05</v>
+        <v>-1.3480168463239126e-05</v>
       </c>
       <c r="AG33">
-        <v>0.00014619121712923053</v>
+        <v>0.00014619121712923123</v>
       </c>
       <c r="AH33">
-        <v>0.0024010981295976529</v>
+        <v>0.0024010981295976537</v>
       </c>
       <c r="AI33">
-        <v>0.00024089133971755663</v>
+        <v>0.00024089133971756486</v>
       </c>
     </row>
     <row r="34">
@@ -3929,103 +3929,103 @@
         <v>-1.5822168062419928</v>
       </c>
       <c r="C34">
-        <v>-7.2034827626274e-05</v>
+        <v>-7.2034827626278066e-05</v>
       </c>
       <c r="D34">
-        <v>-0.0029610538351407139</v>
+        <v>-0.0029610538351408063</v>
       </c>
       <c r="E34">
-        <v>-0.0024047977311919084</v>
+        <v>-0.0024047977311919999</v>
       </c>
       <c r="F34">
-        <v>-0.0020326920215607788</v>
+        <v>-0.0020326920215608581</v>
       </c>
       <c r="G34">
-        <v>-0.0029729672163784247</v>
+        <v>-0.0029729672163785214</v>
       </c>
       <c r="H34">
-        <v>-0.0028559799727096713</v>
+        <v>-0.0028559799727097693</v>
       </c>
       <c r="I34">
-        <v>-0.0024133870012868893</v>
+        <v>-0.0024133870012869878</v>
       </c>
       <c r="J34">
-        <v>-0.002582096142993707</v>
+        <v>-0.0025820961429938089</v>
       </c>
       <c r="K34">
-        <v>-0.0040142065628919503</v>
+        <v>-0.0040142065628920171</v>
       </c>
       <c r="L34">
-        <v>-0.0036131444182356887</v>
+        <v>-0.0036131444182357572</v>
       </c>
       <c r="M34">
-        <v>-0.00015965131485163437</v>
+        <v>-0.00015965131485163692</v>
       </c>
       <c r="N34">
-        <v>-0.00082028153442178608</v>
+        <v>-0.00082028153442179996</v>
       </c>
       <c r="O34">
-        <v>-0.0011770786664807337</v>
+        <v>-0.0011770786664807545</v>
       </c>
       <c r="P34">
-        <v>-0.007646923409067169</v>
+        <v>-0.0076469234090673632</v>
       </c>
       <c r="Q34">
-        <v>-0.0074153616530795467</v>
+        <v>-0.0074153616530797445</v>
       </c>
       <c r="R34">
-        <v>-0.0076541926183776501</v>
+        <v>-0.007654192618377853</v>
       </c>
       <c r="S34">
-        <v>-0.0080109756220309476</v>
+        <v>-0.0080109756220311541</v>
       </c>
       <c r="T34">
-        <v>-0.00073223072105569578</v>
+        <v>-0.00073223072105571747</v>
       </c>
       <c r="U34">
-        <v>-0.0036109294228694145</v>
+        <v>-0.0036109294228694813</v>
       </c>
       <c r="V34">
-        <v>-0.0044241714089441721</v>
+        <v>-0.0044241714089442597</v>
       </c>
       <c r="W34">
-        <v>-0.0053221193019862469</v>
+        <v>-0.0053221193019863666</v>
       </c>
       <c r="X34">
-        <v>0.00018792114322453663</v>
+        <v>0.0001879211432245401</v>
       </c>
       <c r="Y34">
-        <v>-0.00018355116897700159</v>
+        <v>-0.00018355116897699833</v>
       </c>
       <c r="Z34">
-        <v>-0.0030368046871220981</v>
+        <v>-0.0030368046871221436</v>
       </c>
       <c r="AA34">
-        <v>-0.0029087018043451578</v>
+        <v>-0.0029087018043451977</v>
       </c>
       <c r="AB34">
-        <v>-0.0028667674330144039</v>
+        <v>-0.0028667674330144456</v>
       </c>
       <c r="AC34">
-        <v>-0.0028181773427799263</v>
+        <v>-0.0028181773427799692</v>
       </c>
       <c r="AD34">
-        <v>-0.0030305872269813412</v>
+        <v>-0.003030587226981382</v>
       </c>
       <c r="AE34">
-        <v>-0.0028833015366855784</v>
+        <v>-0.00288330153668562</v>
       </c>
       <c r="AF34">
-        <v>-0.00011321363707010669</v>
+        <v>-0.00011321363707010979</v>
       </c>
       <c r="AG34">
-        <v>7.4687898885440079e-06</v>
+        <v>7.4687898885519226e-06</v>
       </c>
       <c r="AH34">
-        <v>0.00024089133971755663</v>
+        <v>0.00024089133971756486</v>
       </c>
       <c r="AI34">
-        <v>0.019747248539181292</v>
+        <v>0.019747248539181771</v>
       </c>
     </row>
   </sheetData>

</xml_diff>